<commit_message>
Restore AI readiness proof lane
</commit_message>
<xml_diff>
--- a/outputs/full-v2-tracker/dayof-full-v2-milestone-tracker.xlsx
+++ b/outputs/full-v2-tracker/dayof-full-v2-milestone-tracker.xlsx
@@ -616,11 +616,6 @@
           <t>DayOf Full V2 Milestone Tracker</t>
         </is>
       </c>
-      <c r="B1" s="13" t="n"/>
-      <c r="C1" s="13" t="n"/>
-      <c r="D1" s="13" t="n"/>
-      <c r="E1" s="13" t="n"/>
-      <c r="F1" s="13" t="n"/>
       <c r="G1" s="23" t="n"/>
       <c r="H1" s="23" t="n"/>
       <c r="I1" s="23" t="n"/>
@@ -888,12 +883,12 @@
       </c>
       <c r="B13" s="43" t="inlineStr">
         <is>
-          <t>2026-05-28 04:57 PM PT</t>
+          <t>2026-05-28 05:51 PM PT</t>
         </is>
       </c>
       <c r="C13" s="13" t="inlineStr">
         <is>
-          <t>Tracker queue refreshed from Exit Bar, Master Milestones, Micro Milestones, QA Gates, and audit findings.</t>
+          <t>Tracker refreshed after restoring ai-product-readiness proof and narrowing browser AI to deterministic/server-only key paths.</t>
         </is>
       </c>
       <c r="D13" s="13" t="n"/>
@@ -6295,7 +6290,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E7"/>
+  <dimension ref="A1:E8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -6491,6 +6486,33 @@
       <c r="E7" s="13" t="inlineStr">
         <is>
           <t>Use V2 Closeout Queue rank order for the next implementation/proof batches; update gates only when evidence is green or claims are narrowed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2026-05-28 05:51 PM PT</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>AI proof restoration</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Restored ai-product-readiness proof and removed browser-side Vite OpenAI key path.</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>npm run proof:v1:ai-product-readiness passed 7/7; src/lib/openai.ts now reads OPENAI_API_KEY / OPENAI_MODEL only, so Quick Start and draft generation prove deterministic fallback instead of browser-key AI.</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Keep V2-G07 In progress until cross-surface claims review and any retained server-backed AI lanes are fully reconciled.</t>
         </is>
       </c>
     </row>
@@ -6527,15 +6549,6 @@
           <t>DayOf V2 Closeout Queue</t>
         </is>
       </c>
-      <c r="B1" s="13" t="n"/>
-      <c r="C1" s="13" t="n"/>
-      <c r="D1" s="13" t="n"/>
-      <c r="E1" s="13" t="n"/>
-      <c r="F1" s="13" t="n"/>
-      <c r="G1" s="13" t="n"/>
-      <c r="H1" s="13" t="n"/>
-      <c r="I1" s="13" t="n"/>
-      <c r="J1" s="13" t="n"/>
     </row>
     <row r="2">
       <c r="A2" s="13" t="inlineStr">
@@ -6660,17 +6673,17 @@
       </c>
       <c r="G5" s="46" t="inlineStr">
         <is>
-          <t>A release gate currently fails before testing behavior because proof scripts referenced by package.json are missing; proof board freshness is also stale.</t>
+          <t>Release-proof drift still exists, but one concrete blocker is repaired: ai-product-readiness is back as a real proof command. Board freshness and any remaining stale proof wiring still need cleanup.</t>
         </is>
       </c>
       <c r="H5" s="46" t="inlineStr">
         <is>
-          <t>Restore/replace stale proof scripts or remove/narrow obsolete gates, refresh BACKLOG current-state truth, and record the exact release-proof contract.</t>
+          <t>Keep reconciling stale proof aliases, refresh BACKLOG current-state truth, and record the exact release-proof contract.</t>
         </is>
       </c>
       <c r="I5" s="46" t="inlineStr">
         <is>
-          <t>proof script inventory clean or explicitly narrowed; proof:v1:board:freshness green; AI readiness gate restored/narrowed.</t>
+          <t>ai-product-readiness green; proof:v1:board:freshness still needs to go green; remaining stale proof references reconciled or narrowed.</t>
         </is>
       </c>
       <c r="J5" s="46" t="inlineStr">
@@ -7010,17 +7023,17 @@
       </c>
       <c r="G12" s="46" t="inlineStr">
         <is>
-          <t>AI readiness proof is missing and V2 copy cannot overclaim model-backed intelligence.</t>
+          <t>The proof command is restored, and browser AI is now narrowed away from Vite-exposed keys. The gate is still open until claims and any retained server-backed lanes are fully reconciled.</t>
         </is>
       </c>
       <c r="H12" s="46" t="inlineStr">
         <is>
-          <t>Restore AI readiness proof, classify model-backed/deterministic/non-AI lanes, scan copy, and prove safe fallbacks/grounding where applicable.</t>
+          <t>Use restored ai-product-readiness proof, then finish claims-matrix review and any retained server-backed lane proof.</t>
         </is>
       </c>
       <c r="I12" s="46" t="inlineStr">
         <is>
-          <t>AI readiness proof green or explicit narrowed claims; no provider/token/model/spend language on customer surfaces.</t>
+          <t>2026-05-28 npm run proof:v1:ai-product-readiness passed 7/7 with deterministic fallback rails, assisted-copy assertions, public-boundary tests, and photo/vault safety checks.</t>
         </is>
       </c>
       <c r="J12" s="46" t="inlineStr">
@@ -7361,11 +7374,6 @@
           <t>Testing vs Build Split</t>
         </is>
       </c>
-      <c r="B1" s="13" t="n"/>
-      <c r="C1" s="13" t="n"/>
-      <c r="D1" s="13" t="n"/>
-      <c r="E1" s="13" t="n"/>
-      <c r="F1" s="13" t="n"/>
     </row>
     <row r="2">
       <c r="A2" s="13" t="inlineStr">
@@ -7673,17 +7681,17 @@
       </c>
       <c r="D12" s="46" t="inlineStr">
         <is>
-          <t>AI readiness proof script is missing; AI claims must be classified.</t>
+          <t>AI readiness proof is restored and browser OpenAI key exposure is removed, but claims still need final cross-surface narrowing/readback.</t>
         </is>
       </c>
       <c r="E12" s="46" t="inlineStr">
         <is>
-          <t>AI readiness proof green or claims narrowed to deterministic/non-AI lanes.</t>
+          <t>Local AI readiness proof green plus final claims review and any retained server-backed lane proof.</t>
         </is>
       </c>
       <c r="F12" s="46" t="inlineStr">
         <is>
-          <t>Restore proof and run claims matrix.</t>
+          <t>Run claims matrix review and keep secure-model/live proof attached only to truly retained server-backed routes.</t>
         </is>
       </c>
     </row>
@@ -7852,12 +7860,6 @@
           <t>DayOf V2 Consumer-Ready Exit Bar</t>
         </is>
       </c>
-      <c r="B1" s="13" t="n"/>
-      <c r="C1" s="13" t="n"/>
-      <c r="D1" s="13" t="n"/>
-      <c r="E1" s="13" t="n"/>
-      <c r="F1" s="13" t="n"/>
-      <c r="G1" s="13" t="n"/>
       <c r="H1" s="13" t="n"/>
       <c r="I1" s="13" t="n"/>
       <c r="J1" s="13" t="n"/>
@@ -7874,11 +7876,6 @@
           <t>Do not call this V2 done because rows are marked Done. Call it V2 only when every must-pass gate below is green, every P0/P1 consumer blocker is closed, and any deferral has matching narrowed product claims.</t>
         </is>
       </c>
-      <c r="C2" s="13" t="n"/>
-      <c r="D2" s="13" t="n"/>
-      <c r="E2" s="13" t="n"/>
-      <c r="F2" s="13" t="n"/>
-      <c r="G2" s="13" t="n"/>
       <c r="H2" s="13" t="n"/>
       <c r="I2" s="13" t="n"/>
       <c r="J2" s="13" t="n"/>
@@ -7895,11 +7892,6 @@
           <t>A real couple can onboard, build, publish/share, manage guests, message, collect photos, use registry/vault, and hand the experience to guests without us explaining caveats in person.</t>
         </is>
       </c>
-      <c r="C3" s="13" t="n"/>
-      <c r="D3" s="13" t="n"/>
-      <c r="E3" s="13" t="n"/>
-      <c r="F3" s="13" t="n"/>
-      <c r="G3" s="13" t="n"/>
       <c r="H3" s="13" t="n"/>
       <c r="I3" s="13" t="n"/>
       <c r="J3" s="13" t="n"/>
@@ -8350,27 +8342,27 @@
       </c>
       <c r="G12" s="38" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="H12" s="51" t="inlineStr">
         <is>
-          <t>Proof infra + narrowing</t>
+          <t>Proof restored</t>
         </is>
       </c>
       <c r="I12" s="13" t="inlineStr">
         <is>
-          <t>No. Restore/replace AI readiness proof first.</t>
+          <t>Partly: local AI readiness proof is green again.</t>
         </is>
       </c>
       <c r="J12" s="13" t="inlineStr">
         <is>
-          <t>Classify AI lanes as model-backed, deterministic, or non-AI; prove or narrow claims.</t>
+          <t>Cross-surface AI claims matrix and any retained server-backed lanes still need human readback and live/server proof where applicable.</t>
         </is>
       </c>
       <c r="K12" s="13" t="inlineStr">
         <is>
-          <t>npm run proof:v1:ai-product-readiness currently points at a missing script.</t>
+          <t>2026-05-28 restored npm run proof:v1:ai-product-readiness (7/7). Browser OpenAI key path removed; Quick Start and draft generation now prove deterministic fallback rails.</t>
         </is>
       </c>
     </row>
@@ -8769,7 +8761,7 @@
       </c>
       <c r="K19" s="13" t="inlineStr">
         <is>
-          <t>proof:v1:board:freshness is stale; package script inventory found missing proof files.</t>
+          <t>Proof infra improved: ai-product-readiness restored on 2026-05-28, but proof:v1:board:freshness is still stale and broader proof-script drift still needs reconciliation.</t>
         </is>
       </c>
     </row>
@@ -10682,7 +10674,7 @@
       </c>
       <c r="F22" s="23" t="inlineStr">
         <is>
-          <t>AI copy may be safer in places, but the AI product contract is not green: proof:v1:ai-product-readiness currently points at a missing script and AI lanes still need classification/narrowing.</t>
+          <t>Local AI readiness proof is restored and green again, and browser-side OpenAI key usage is removed in favor of deterministic fallback/server-only key paths. The AI gate remains In progress until cross-surface claims and any retained server-backed lanes are fully reconciled.</t>
         </is>
       </c>
       <c r="G22" s="23" t="inlineStr">
@@ -10910,7 +10902,7 @@
       </c>
       <c r="F26" s="23" t="inlineStr">
         <is>
-          <t>Tracker/proof reconciliation is now explicitly underway, but proof infrastructure is stale: proof board freshness fails and multiple package proof commands point at absent scripts.</t>
+          <t>Tracker/proof reconciliation is still in progress. ai-product-readiness is restored, but proof board freshness remains stale and the broader release-proof contract still needs cleanup.</t>
         </is>
       </c>
       <c r="G26" s="23" t="inlineStr">

</xml_diff>

<commit_message>
Refresh proof board launch truth
</commit_message>
<xml_diff>
--- a/outputs/full-v2-tracker/dayof-full-v2-milestone-tracker.xlsx
+++ b/outputs/full-v2-tracker/dayof-full-v2-milestone-tracker.xlsx
@@ -883,12 +883,12 @@
       </c>
       <c r="B13" s="43" t="inlineStr">
         <is>
-          <t>2026-05-28 05:51 PM PT</t>
+          <t>2026-05-28 05:54 PM PT</t>
         </is>
       </c>
       <c r="C13" s="13" t="inlineStr">
         <is>
-          <t>Tracker refreshed after restoring ai-product-readiness proof and narrowing browser AI to deterministic/server-only key paths.</t>
+          <t>Tracker refreshed after proof-board freshness returned to green; release-proof cleanup remains in progress.</t>
         </is>
       </c>
       <c r="D13" s="13" t="n"/>
@@ -6290,7 +6290,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E8"/>
+  <dimension ref="A1:E9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -6513,6 +6513,33 @@
       <c r="E8" t="inlineStr">
         <is>
           <t>Keep V2-G07 In progress until cross-surface claims review and any retained server-backed AI lanes are fully reconciled.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2026-05-28 05:54 PM PT</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Proof board freshness</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Refreshed BACKLOG current-state truth so the proof board is fresh again.</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>`npm run proof:v1:board:freshness` passed and `npm run proof:v1:board:md` rendered cleanly after updating the BACKLOG current-state block without changing deployed launch claims.</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Keep V2-G14 In progress until the broader release-proof contract and any remaining stale proof references are reconciled.</t>
         </is>
       </c>
     </row>
@@ -6673,17 +6700,17 @@
       </c>
       <c r="G5" s="46" t="inlineStr">
         <is>
-          <t>Release-proof drift still exists, but one concrete blocker is repaired: ai-product-readiness is back as a real proof command. Board freshness and any remaining stale proof wiring still need cleanup.</t>
+          <t>The proof surface is healthier now: ai-product-readiness is restored, and proof-board freshness is green again. The item still stays open until the remaining release-proof contract is reconciled.</t>
         </is>
       </c>
       <c r="H5" s="46" t="inlineStr">
         <is>
-          <t>Keep reconciling stale proof aliases, refresh BACKLOG current-state truth, and record the exact release-proof contract.</t>
+          <t>Keep reconciling any stale proof aliases, keep BACKLOG current-state truth fresh, and record the exact release-proof contract the closeout relies on.</t>
         </is>
       </c>
       <c r="I5" s="46" t="inlineStr">
         <is>
-          <t>ai-product-readiness green; proof:v1:board:freshness still needs to go green; remaining stale proof references reconciled or narrowed.</t>
+          <t>2026-05-28 `proof:v1:ai-product-readiness` PASS 7/7, `proof:v1:board:freshness` PASS, and `proof:v1:board:md` PASS.</t>
         </is>
       </c>
       <c r="J5" s="46" t="inlineStr">
@@ -7649,17 +7676,17 @@
       </c>
       <c r="D11" s="46" t="inlineStr">
         <is>
-          <t>Proof commands are stale/missing and proof board freshness fails.</t>
+          <t>The biggest freshness blocker is fixed: board freshness now passes, and ai-product-readiness is restored. Remaining work is narrower release-proof contract reconciliation.</t>
         </is>
       </c>
       <c r="E11" s="46" t="inlineStr">
         <is>
-          <t>Missing proof references resolved; BACKLOG truth fresh; proof bundle defined.</t>
+          <t>Board freshness green, proof board render green, and any remaining relied-on proof aliases reconciled or honestly narrowed.</t>
         </is>
       </c>
       <c r="F11" s="46" t="inlineStr">
         <is>
-          <t>Repair proof scripts or narrow obsolete gates.</t>
+          <t>Continue release-proof cleanup from the closeout queue until no stale relied-on proof lane remains.</t>
         </is>
       </c>
     </row>
@@ -8746,22 +8773,22 @@
       </c>
       <c r="H19" s="51" t="inlineStr">
         <is>
-          <t>Proof infra + release docs</t>
+          <t>Proof infra in progress</t>
         </is>
       </c>
       <c r="I19" s="13" t="inlineStr">
         <is>
-          <t>No. Release proof tooling/truth must be repaired first.</t>
+          <t>Partly: board freshness and markdown board are green again.</t>
         </is>
       </c>
       <c r="J19" s="13" t="inlineStr">
         <is>
-          <t>Repair stale/missing proof scripts, refresh BACKLOG truth, reconcile tracker/proof docs, and write rollback plan.</t>
+          <t>Broader release-proof contract still needs reconciliation so every relied-on proof lane is real, current, and honestly scoped.</t>
         </is>
       </c>
       <c r="K19" s="13" t="inlineStr">
         <is>
-          <t>Proof infra improved: ai-product-readiness restored on 2026-05-28, but proof:v1:board:freshness is still stale and broader proof-script drift still needs reconciliation.</t>
+          <t>2026-05-28 `npm run proof:v1:board:freshness` PASS and `npm run proof:v1:board:md` PASS after refreshing BACKLOG.md current-state block. ai-product-readiness was already restored in the prior batch.</t>
         </is>
       </c>
     </row>
@@ -10902,7 +10929,7 @@
       </c>
       <c r="F26" s="23" t="inlineStr">
         <is>
-          <t>Tracker/proof reconciliation is still in progress. ai-product-readiness is restored, but proof board freshness remains stale and the broader release-proof contract still needs cleanup.</t>
+          <t>Tracker/proof reconciliation is still in progress, but two concrete proof-infra gaps are repaired: ai-product-readiness is restored and proof-board freshness is green again. The remaining release-proof contract cleanup is narrower and still open.</t>
         </is>
       </c>
       <c r="G26" s="23" t="inlineStr">

</xml_diff>

<commit_message>
Close first-session smoke gate
</commit_message>
<xml_diff>
--- a/outputs/full-v2-tracker/dayof-full-v2-milestone-tracker.xlsx
+++ b/outputs/full-v2-tracker/dayof-full-v2-milestone-tracker.xlsx
@@ -1041,7 +1041,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E11"/>
+  <dimension ref="A1:E12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1338,6 +1338,33 @@
       <c r="E11" t="inlineStr">
         <is>
           <t>Mark V2-G03 and V2-03.06 done, then keep Builder V2 follow-up limited to public runtime/template parity and legacy photo-polish work.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2026-05-28 07:08 PM PT</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>First-session couple path</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Closed the first-session smoke lane locally.</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>2026-05-28 local PASS: PLAYWRIGHT_BASE_URL=http://127.0.0.1:4173 npm run test:e2e:first-session passed 7/7, covering signed-out homepage/product/signup/quick-start entry truth plus signed-local desktop/mobile celebration, quick-start, guests-to-photos, review/share, and builder-guide continuation.</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Mark V2-G02 and V2-01.05 done, keep V2-G01 honestly in progress until the broader claims matrix and later-surface narrowing are finished.</t>
         </is>
       </c>
     </row>
@@ -1370,7 +1397,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-05-28 06:29 PM PT</t>
+          <t>2026-05-28 07:08 PM PT</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -1562,27 +1589,27 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>First-session couple path smoke</t>
+          <t>Closed 2026-05-28: First-session couple path smoke</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>The first five minutes decide whether V2 feels real. Tracker says proof is still open.</t>
+          <t>Signed-out and signed-local desktop/mobile first-session browser proof is now attached for the first five minutes.</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>Run signed-out and signed-in desktop/mobile first-session smoke from Home/Product/Signup/QuickStart through build/publish/share next step.</t>
+          <t>Closed in this batch: proved public entry truth from Home/Product/Signup into quick-start preview, then signed-local celebration -&gt; quick-start -&gt; guests -&gt; photos -&gt; overview/share -&gt; builder-guide continuation on desktop and mobile.</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>A new couple reaches a useful setup/build/publish state without internal language or fake readiness claims.</t>
+          <t>2026-05-28 local PASS: PLAYWRIGHT_BASE_URL=http://127.0.0.1:4173 npm run test:e2e:first-session passed 7/7, covering signed-out homepage/product/signup/quick-start entry truth plus signed-local desktop/mobile celebration, quick-start, guests-to-photos, review/share, and builder-guide continuation.</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>Any maze/dead-end/overclaim failure becomes a focused patch.</t>
+          <t>Keep broader product-truth narrowing under V2-G01 and runtime/template work under later gates; do not overclaim this smoke as whole-product completion.</t>
         </is>
       </c>
     </row>
@@ -2169,7 +2196,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-05-28 06:29 PM PT</t>
+          <t>2026-05-28 07:08 PM PT</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -2250,7 +2277,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Can close if testing passes</t>
+          <t>Closed 2026-05-28</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -2265,17 +2292,17 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Implementation may be close; proof is missing.</t>
+          <t>The missing first-session proof is now attached locally across signed-out entry and signed-local desktop/mobile continuation.</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Signed-out/in desktop/mobile smoke reaches useful setup/build/publish path without overclaim.</t>
+          <t>Closed: first-session smoke reaches useful setup, build, review/share, and builder-guide next steps without internal or fake-readiness copy.</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Run first-session smoke and patch only failures.</t>
+          <t>Keep any remaining product-truth work scoped to specific copy or claim lanes instead of reopening the whole funnel.</t>
         </is>
       </c>
     </row>
@@ -2749,7 +2776,7 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>Partly: copy scan can clear shipped surfaces if green.</t>
+          <t>Partly: first-session smoke confirms the current signed-out/in funnel copy and handoffs read as truthful, but broader claims-matrix and later-surface narrowing still remain.</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
@@ -2759,7 +2786,7 @@
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>Audit found no signoff yet; keep status In progress.</t>
+          <t>Audit found no signoff yet; keep status In progress. 2026-05-28 local PASS: PLAYWRIGHT_BASE_URL=http://127.0.0.1:4173 npm run test:e2e:first-session passed 7/7, covering signed-out homepage/product/signup/quick-start entry truth plus signed-local desktop/mobile celebration, quick-start, guests-to-photos, review/share, and builder-guide continuation.</t>
         </is>
       </c>
     </row>
@@ -2796,7 +2823,7 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
@@ -2806,17 +2833,17 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>Yes, if signed-out and signed-in desktop/mobile first-session smoke passes.</t>
+          <t>Done: signed-out and signed-local desktop/mobile first-session browser smoke is now logged for entry, setup, continuation, review/share, and builder-guide next steps.</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>If smoke shows maze/dead-end behavior, patch only the failing handoff/copy.</t>
+          <t>Keep future fixes under specific copy or handoff defects; do not reopen G02 unless the first-session path itself regresses.</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>Tracker says first-session browser proof still open.</t>
+          <t>2026-05-28 local PASS: PLAYWRIGHT_BASE_URL=http://127.0.0.1:4173 npm run test:e2e:first-session passed 7/7, covering signed-out homepage/product/signup/quick-start entry truth plus signed-local desktop/mobile celebration, quick-start, guests-to-photos, review/share, and builder-guide continuation.</t>
         </is>
       </c>
     </row>
@@ -4248,7 +4275,7 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Public entry truth and CTA continuity are materially better across feature pages, templates, trust/product, and support/legal surfaces; first-session browser proof is still open.</t>
+          <t>Public entry truth and CTA continuity are materially better across feature pages, templates, trust/product, and support/legal surfaces; 2026-05-28 signed-out plus signed-local desktop/mobile first-session smoke is now green. Status stays In progress because broader product-truth narrowing and adjacent proof gates remain open.</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -4305,7 +4332,7 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Auth/onboarding continuation and first-session safety are stronger, with clearer setup handoff and safer GuidedSetup/Onboarding recovery copy, but the funnel still needs unified browser proof.</t>
+          <t>Auth/onboarding continuation and first-session safety are stronger, with clearer setup handoff and safer GuidedSetup/Onboarding recovery copy. 2026-05-28 signed-local desktop/mobile first-session smoke is now green across celebration, quick-start, guests, photos, overview/share, and builder-guide continuation, but the broader onboarding spine still stays In progress.</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -5992,12 +6019,12 @@
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>Copy and CTA truth improved across public entry and onboarding, but signed-out and signed-in first-session browser smoke is still open.</t>
+          <t>2026-05-28 signed-out and signed-local desktop/mobile first-session browser smoke passed from Home/Product/Signup into quick-start preview and onward through celebration, quick-start, guests, photos, overview/share, and builder-guide next steps without fake readiness copy.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Advance public V2 runtime proof lane
</commit_message>
<xml_diff>
--- a/outputs/full-v2-tracker/dayof-full-v2-milestone-tracker.xlsx
+++ b/outputs/full-v2-tracker/dayof-full-v2-milestone-tracker.xlsx
@@ -1041,7 +1041,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E12"/>
+  <dimension ref="A1:E13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1365,6 +1365,33 @@
       <c r="E12" t="inlineStr">
         <is>
           <t>Mark V2-G02 and V2-01.05 done, keep V2-G01 honestly in progress until the broader claims matrix and later-surface narrowing are finished.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>2026-05-28 07:31 PM PT</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Public V2 runtime parity</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Moved the public V2/runtime lane from Not started to active proof-backed work.</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>2026-05-28 local PASS: npm run proof:v1:public-v2-runtime passed with 59 focused V2/public runtime tests and 4/4 public-site-quality Playwright checks on localhost. The lane now explicitly proves V2 document adaptation, public boundary stripping, canonical row identity, desktop/mobile guest quality, preview-chrome suppression, and current template-variant fallback normalization.</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Keep G04 and the queue item open until representative template visual parity is proven beyond the canonical runtime lane.</t>
         </is>
       </c>
     </row>
@@ -1397,7 +1424,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-05-28 07:08 PM PT</t>
+          <t>2026-05-28 07:31 PM PT</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -1644,7 +1671,7 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>Exit Bar marks public V2 runtime parity Not started, so this cannot close by testing alone.</t>
+          <t>Public runtime parity is now actively proven in part: a dedicated local proof lane exists and is green, but the full template visual matrix and broader representative V2 doc set are still open.</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
@@ -1654,12 +1681,12 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>Runtime tests, template matrix, visual proof set, mobile proof, and no private leaks.</t>
+          <t>2026-05-28 local PASS: npm run proof:v1:public-v2-runtime passed with 59 focused V2/public runtime tests and 4/4 public-site-quality Playwright checks on localhost. The lane now explicitly proves V2 document adaptation, public boundary stripping, canonical row identity, desktop/mobile guest quality, preview-chrome suppression, and current template-variant fallback normalization.</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>Do not call Builder V2 complete if public V2 output is only schema-compatible or visually placeholder.</t>
+          <t>Keep this queue item open until representative V2 templates and public pages have broader visual/matrix proof, not just canonical demo/runtime checks.</t>
         </is>
       </c>
     </row>
@@ -2196,7 +2223,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-05-28 07:08 PM PT</t>
+          <t>2026-05-28 07:31 PM PT</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -2420,17 +2447,17 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Tracker marks this Not started and it is foundational to V2.</t>
+          <t>This has moved from a blank Not started lane to an active proof-backed lane, but it still needs broader representative-template coverage before it can close.</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>V2 docs render polished public desktop/mobile sites with section parity.</t>
+          <t>V2 docs render guest-safe public desktop/mobile sites with explicit runtime proof, no preview leaks, and variant fallback normalization; remaining closure work is the representative template visual matrix.</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Build/prove runtime, template matrix, visual set.</t>
+          <t>Extend the green public-v2-runtime proof from canonical/demo coverage into a broader representative template screenshot matrix.</t>
         </is>
       </c>
     </row>
@@ -2937,7 +2964,7 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
@@ -2947,17 +2974,17 @@
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>No. Tests can expose the gap, but public V2 runtime parity is still marked Not started.</t>
+          <t>In progress: a dedicated public-v2-runtime proof lane is now green locally, covering V2 document adaptation, public boundary stripping, canonical row identity, and desktop/mobile public quality. Representative template visual parity is still open.</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>Build/prove V2 public renderer parity, template visual set, mobile/metadata/leak proof.</t>
+          <t>Finish the representative template/runtime screenshot matrix and any remaining mobile/metadata/leak proof before closing G04.</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>Exit Bar status Not started.</t>
+          <t>2026-05-28 local PASS: npm run proof:v1:public-v2-runtime passed with 59 focused V2/public runtime tests and 4/4 public-site-quality Playwright checks on localhost. The lane now explicitly proves V2 document adaptation, public boundary stripping, canonical row identity, desktop/mobile guest quality, preview-chrome suppression, and current template-variant fallback normalization.</t>
         </is>
       </c>
     </row>
@@ -4441,12 +4468,12 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Template chooser improved; long-tail variant/import compatibility still needs V2-grade proof.</t>
+          <t>Template chooser improved; public template/runtime proof is now active through the new public-v2-runtime lane and variant fallback coverage, but the broader representative-template compatibility and visual matrix still need V2-grade proof.</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -4498,12 +4525,12 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Current public runtime exists, but V2 document runtime parity remains Not started in the tracker and blocks V2 until proven with mobile/template/leak evidence.</t>
+          <t>Public runtime already exists, and 2026-05-28 public-v2-runtime proof is now green locally for V2 document adaptation, guest-safe boundary stripping, canonical row identity, and desktop/mobile public quality. Status stays In progress because the representative template visual matrix and broader parity set are still open.</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -6715,7 +6742,12 @@
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>In progress</t>
+        </is>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>2026-05-28 public runtime proof now includes explicit variant fallback normalization coverage for guest-safe public rendering (hero video -&gt; default, registry luxury -&gt; featured, gallery/story fallbacks), but the full shipped variant matrix remains open.</t>
         </is>
       </c>
     </row>
@@ -7027,12 +7059,12 @@
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="K25" t="inlineStr">
         <is>
-          <t>Audit-derived V2 readiness gap.</t>
+          <t>2026-05-28 local PASS: npm run proof:v1:public-v2-runtime passed with 59 focused V2/public runtime tests and 4/4 public-site-quality Playwright checks on localhost. The lane now explicitly proves V2 document adaptation, public boundary stripping, canonical row identity, desktop/mobile guest quality, preview-chrome suppression, and current template-variant fallback normalization.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Close public V2 template parity gate
</commit_message>
<xml_diff>
--- a/outputs/full-v2-tracker/dayof-full-v2-milestone-tracker.xlsx
+++ b/outputs/full-v2-tracker/dayof-full-v2-milestone-tracker.xlsx
@@ -1041,7 +1041,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E13"/>
+  <dimension ref="A1:E14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1392,6 +1392,33 @@
       <c r="E13" t="inlineStr">
         <is>
           <t>Keep G04 and the queue item open until representative template visual parity is proven beyond the canonical runtime lane.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2026-05-28 07:36 PM PT</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Public V2 runtime parity</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Closed the public V2/runtime parity lane locally.</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>2026-05-28 local PASS: npm run proof:v1:public-v2-runtime now enforces the full public V2/runtime lane: 59 focused V2/public runtime tests, 4/4 public-site-quality Playwright checks, and template-hardening audit green at 35/35 templates passed + distinct and 57/57 strict variants resolved on localhost.</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>Mark queue item 4, V2-G04, V2-04.03, V2-04.04, and V2-05.05 done; keep G13 and the broader whole-product polish matrix open.</t>
         </is>
       </c>
     </row>
@@ -1424,7 +1451,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-05-28 07:31 PM PT</t>
+          <t>2026-05-28 07:36 PM PT</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -1666,27 +1693,27 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Public V2 runtime and template parity</t>
+          <t>Closed 2026-05-28: Public V2 runtime and template parity</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>Public runtime parity is now actively proven in part: a dedicated local proof lane exists and is green, but the full template visual matrix and broader representative V2 doc set are still open.</t>
+          <t>The public V2/runtime lane is now fully proof-backed locally: canonical runtime, desktop/mobile guest quality, no preview leaks, and representative template matrix distinctness all pass.</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>Build/prove V2 public renderer parity, template import/compatibility, visual proof, metadata, mobile, and leak boundaries.</t>
+          <t>Closed in this batch: strengthened proof:v1:public-v2-runtime to enforce the representative template visual matrix, then passed the runtime tests, public-site-quality smoke, 35/35 distinct template audit, and 57/57 strict variant audit.</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>2026-05-28 local PASS: npm run proof:v1:public-v2-runtime passed with 59 focused V2/public runtime tests and 4/4 public-site-quality Playwright checks on localhost. The lane now explicitly proves V2 document adaptation, public boundary stripping, canonical row identity, desktop/mobile guest quality, preview-chrome suppression, and current template-variant fallback normalization.</t>
+          <t>2026-05-28 local PASS: npm run proof:v1:public-v2-runtime now enforces the full public V2/runtime lane: 59 focused V2/public runtime tests, 4/4 public-site-quality Playwright checks, and template-hardening audit green at 35/35 templates passed + distinct and 57/57 strict variants resolved on localhost.</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>Keep this queue item open until representative V2 templates and public pages have broader visual/matrix proof, not just canonical demo/runtime checks.</t>
+          <t>Keep whole-product visual/mobile/a11y review under G13; do not use this closure to imply the entire product polish matrix is finished.</t>
         </is>
       </c>
     </row>
@@ -2223,7 +2250,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-05-28 07:31 PM PT</t>
+          <t>2026-05-28 07:36 PM PT</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -2432,7 +2459,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Not done / needs actual work</t>
+          <t>Closed 2026-05-28</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -2447,17 +2474,17 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>This has moved from a blank Not started lane to an active proof-backed lane, but it still needs broader representative-template coverage before it can close.</t>
+          <t>The lane now has an enforced proof bundle, not just scattered tests: runtime tests, public quality smoke, and representative template distinctness all pass locally.</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>V2 docs render guest-safe public desktop/mobile sites with explicit runtime proof, no preview leaks, and variant fallback normalization; remaining closure work is the representative template visual matrix.</t>
+          <t>Closed: V2 public runtime adaptation, guest-safe boundary stripping, desktop/mobile public quality, preview-chrome suppression, and representative template visual matrix are green locally.</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Extend the green public-v2-runtime proof from canonical/demo coverage into a broader representative template screenshot matrix.</t>
+          <t>Keep later visual/mobile/a11y work scoped to the broader whole-product polish matrix, not this runtime parity lane.</t>
         </is>
       </c>
     </row>
@@ -2964,7 +2991,7 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
@@ -2974,17 +3001,17 @@
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>In progress: a dedicated public-v2-runtime proof lane is now green locally, covering V2 document adaptation, public boundary stripping, canonical row identity, and desktop/mobile public quality. Representative template visual parity is still open.</t>
+          <t>Done: the public V2/runtime lane is now proven locally with enforced runtime tests, desktop/mobile public quality smoke, no preview leaks, canonical row identity, and representative template/variant matrix proof.</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>Finish the representative template/runtime screenshot matrix and any remaining mobile/metadata/leak proof before closing G04.</t>
+          <t>Keep future regressions under targeted runtime/template fixes; do not reopen G04 unless public V2 render parity itself breaks.</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>2026-05-28 local PASS: npm run proof:v1:public-v2-runtime passed with 59 focused V2/public runtime tests and 4/4 public-site-quality Playwright checks on localhost. The lane now explicitly proves V2 document adaptation, public boundary stripping, canonical row identity, desktop/mobile guest quality, preview-chrome suppression, and current template-variant fallback normalization.</t>
+          <t>2026-05-28 local PASS: npm run proof:v1:public-v2-runtime now enforces the full public V2/runtime lane: 59 focused V2/public runtime tests, 4/4 public-site-quality Playwright checks, and template-hardening audit green at 35/35 templates passed + distinct and 57/57 strict variants resolved on localhost.</t>
         </is>
       </c>
     </row>
@@ -6742,12 +6769,12 @@
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>2026-05-28 public runtime proof now includes explicit variant fallback normalization coverage for guest-safe public rendering (hero video -&gt; default, registry luxury -&gt; featured, gallery/story fallbacks), but the full shipped variant matrix remains open.</t>
+          <t>2026-05-28 template-hardening audit passed strict variants 57/57, and public runtime fallback normalization coverage is locked by proof:v1:public-v2-runtime plus SiteView variant-normalization tests.</t>
         </is>
       </c>
     </row>
@@ -6799,7 +6826,12 @@
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>2026-05-28 template-hardening audit passed 35/35 representative templates with distinct section hashes and required public tokens on localhost; no template leak hits were found.</t>
         </is>
       </c>
     </row>
@@ -7059,12 +7091,12 @@
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K25" t="inlineStr">
         <is>
-          <t>2026-05-28 local PASS: npm run proof:v1:public-v2-runtime passed with 59 focused V2/public runtime tests and 4/4 public-site-quality Playwright checks on localhost. The lane now explicitly proves V2 document adaptation, public boundary stripping, canonical row identity, desktop/mobile guest quality, preview-chrome suppression, and current template-variant fallback normalization.</t>
+          <t>2026-05-28 local PASS: npm run proof:v1:public-v2-runtime now enforces the full public V2/runtime lane: 59 focused V2/public runtime tests, 4/4 public-site-quality Playwright checks, and template-hardening audit green at 35/35 templates passed + distinct and 57/57 strict variants resolved on localhost.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Close guest journey proof gate
</commit_message>
<xml_diff>
--- a/outputs/full-v2-tracker/dayof-full-v2-milestone-tracker.xlsx
+++ b/outputs/full-v2-tracker/dayof-full-v2-milestone-tracker.xlsx
@@ -1041,7 +1041,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E14"/>
+  <dimension ref="A1:E15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1419,6 +1419,33 @@
       <c r="E14" t="inlineStr">
         <is>
           <t>Mark queue item 4, V2-G04, V2-04.03, V2-04.04, and V2-05.05 done; keep G13 and the broader whole-product polish matrix open.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>2026-05-28 06:47 PM PT</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Guest journey proof</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Unified mobile guest-path proof is now green locally.</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>PLAYWRIGHT_BASE_URL=http://127.0.0.1:4173 npm run proof:v1:guest-journey passed with 13/13 unit tests and 2/2 Playwright checks across public site, RSVP entry, contact update, photo upload, registry, vault, and stale/incomplete-link recovery.</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>Keep photo/vault delight depth and whole-product visual polish under V2-15.05 and V2-24.05; do not reopen G05 unless the guest path regresses.</t>
         </is>
       </c>
     </row>
@@ -1451,7 +1478,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-05-28 07:36 PM PT</t>
+          <t>2026-05-28 06:47 PM PT</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -1743,27 +1770,27 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Zero-friction guest journey proof</t>
+          <t>Closed 2026-05-28: Zero-friction guest journey proof</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>Guest flows are strong in pieces, but tracker still lacks unified guest happy-path proof.</t>
+          <t>Local guest proof now covers public site, RSVP entry, contact update, photo upload, registry, vault, and stale/incomplete-link recovery on mobile without guest-facing internal wording.</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>Run invite-linked mobile guest proof covering RSVP, schedule/travel, photo upload, contact update, registry, vault, and return-later behavior.</t>
+          <t>Closed in this batch: added proof:v1:guest-journey, guest-happy-path-mobile Playwright smoke, and deterministic copy/unit coverage for guest journey, RSVP/contact recovery, and vault continuity paths.</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>Guest happy path and stale/invalid link recovery pass without token/debug/provider/ops wording.</t>
+          <t>2026-05-28 local PASS: PLAYWRIGHT_BASE_URL=http://127.0.0.1:4173 npm run proof:v1:guest-journey passed with 13/13 unit tests and 2/2 Playwright checks covering public site, RSVP entry, contact update, photo upload, registry, vault, and stale/incomplete-link recovery.</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>Patch failures in the specific guest surface before marking G05 done.</t>
+          <t>Keep upload delight depth and whole-product visual polish under V2-15.05 and V2-24.05; do not overclaim those from this guest-path proof.</t>
         </is>
       </c>
     </row>
@@ -2232,7 +2259,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F16"/>
+  <dimension ref="A1:F17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2250,7 +2277,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-05-28 07:36 PM PT</t>
+          <t>2026-05-28 06:47 PM PT</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -2677,6 +2704,38 @@
       <c r="F16" t="inlineStr">
         <is>
           <t>Run visual/mobile matrix after core gates stabilize.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Closed 2026-05-28</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Zero-friction guest journey proof</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>V2-G05</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>The missing unified guest-path proof is now attached locally across mobile public, RSVP entry, contact, upload, registry, vault, and stale/incomplete recovery.</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>Closed: proof:v1:guest-journey is green with 13/13 unit tests and 2/2 Playwright checks, and guest-facing copy stays free of token/debug/provider/internal wording.</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>Keep deeper photo/vault delight and whole-product visual polish under V2-15.05 and V2-24.05 instead of reopening this gate.</t>
         </is>
       </c>
     </row>
@@ -2729,7 +2788,6 @@
         </is>
       </c>
     </row>
-    <row r="4"/>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
@@ -3048,7 +3106,7 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
@@ -3058,17 +3116,17 @@
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>Partly: run guest happy-path mobile/browser proof to discover remaining failures.</t>
+          <t>Yes: local guest-journey proof is green and stale/incomplete-link recovery stays guest-safe on mobile.</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>Patch any token continuity, stale-link recovery, public route, or guest-safe copy failures.</t>
+          <t>Keep deeper photo/vault delight and whole-product visual polish under their separate gates, not under G05.</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>Exit Bar In progress; micro V2-06.* mostly Not started.</t>
+          <t>2026-05-28 local PASS: PLAYWRIGHT_BASE_URL=http://127.0.0.1:4173 npm run proof:v1:guest-journey passed with 13/13 unit tests and 2/2 Playwright checks across public site, RSVP entry, contact update, photo upload, registry, vault, and stale/incomplete-link recovery.</t>
         </is>
       </c>
     </row>
@@ -4609,12 +4667,12 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Guest journey companion is strong; all guest tools need end-to-end V2 continuity proof.</t>
+          <t>2026-05-28 local guest-journey proof is green across public site, RSVP entry, contact update, photo upload, registry, vault, and stale/incomplete-link recovery. Status stays In progress because adjacent guest-depth items in guests/photos/memory still remain outside the core proof lane.</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -7148,7 +7206,12 @@
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>In progress</t>
+        </is>
+      </c>
+      <c r="K26" t="inlineStr">
+        <is>
+          <t>2026-05-28 local PASS: guestJourney unit coverage plus guest-happy-path mobile proof confirm contextual next-step links across contact/photo/vault and stable journey-link generation from RSVP-oriented contexts.</t>
         </is>
       </c>
     </row>
@@ -7200,7 +7263,12 @@
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>In progress</t>
+        </is>
+      </c>
+      <c r="K27" t="inlineStr">
+        <is>
+          <t>2026-05-28 local PASS: stale/incomplete recovery is guest-safe on /events, /guest-contact/:token, and /vault/:siteSlug/:year; broader live token continuity still rides with RSVP/contact live data lanes.</t>
         </is>
       </c>
     </row>
@@ -7252,7 +7320,12 @@
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="K28" t="inlineStr">
+        <is>
+          <t>2026-05-28 local PASS: proof:v1:guest-journey Playwright 2/2 covered mobile public site, RSVP entry, contact update, photo upload, registry, vault, and recovery routes without critical layout blockers.</t>
         </is>
       </c>
     </row>
@@ -7304,7 +7377,12 @@
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="K29" t="inlineStr">
+        <is>
+          <t>2026-05-28 local PASS: guest-happy-path-mobile asserts no invite_token/provider/debug/internal wording across guest path and stale/incomplete recovery surfaces.</t>
         </is>
       </c>
     </row>
@@ -7356,12 +7434,12 @@
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K30" t="inlineStr">
         <is>
-          <t>Audit-derived V2 readiness gap.</t>
+          <t>2026-05-28 local PASS: proof:v1:guest-journey passed with 13/13 unit tests and 2/2 Playwright checks, closing the unified mobile guest happy-path proof lane.</t>
         </is>
       </c>
     </row>
@@ -8275,7 +8353,12 @@
       </c>
       <c r="J47" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>In progress</t>
+        </is>
+      </c>
+      <c r="K47" t="inlineStr">
+        <is>
+          <t>2026-05-28 V2 successor proof:v1:guest-journey now covers the public RSVP entry path plus guest continuity/recovery. Legacy guests-rsvp-ops proof remains a separate lane.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Close registry public parity gate
</commit_message>
<xml_diff>
--- a/outputs/full-v2-tracker/dayof-full-v2-milestone-tracker.xlsx
+++ b/outputs/full-v2-tracker/dayof-full-v2-milestone-tracker.xlsx
@@ -1041,7 +1041,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E15"/>
+  <dimension ref="A1:E16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1446,6 +1446,33 @@
       <c r="E15" t="inlineStr">
         <is>
           <t>Keep photo/vault delight depth and whole-product visual polish under V2-15.05 and V2-24.05; do not reopen G05 unless the guest path regresses.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2026-05-28 06:53 PM PT</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Registry parity proof</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Dashboard/public registry trust is now green locally for the parity lane.</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>npm run proof:v1:registry-public-parity passed with 105/105 tests across registryPublicParity, registryService, RegistrySection, and RegistryDashboardRouteContent, covering purchased, hidden, fund-share, and thank-you-relevant truth.</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>Keep live owner/public runtime verification and broader registry operating-system proof under the remaining registry lanes; do not overclaim live write/read from this local parity closure.</t>
         </is>
       </c>
     </row>
@@ -1478,7 +1505,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-05-28 06:47 PM PT</t>
+          <t>2026-05-28 06:53 PM PT</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -1820,27 +1847,27 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Registry public parity proof</t>
+          <t>Closed 2026-05-28: Registry public parity proof</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>Registry dashboard work is advanced, but public purchased/hidden/fund/thank-you parity remains open.</t>
+          <t>Registry dashboard/public trust is now backed by a focused parity proof that compares guest-visible public registry truth against dashboard-derived purchased, hidden, fund, and thank-you state.</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>Run public registry parity proof and focused registry suite.</t>
+          <t>Closed in this batch: added proof:v1:registry-public-parity and a dedicated parity suite covering public guest visibility, hidden purchased items, fund share readiness, and thank-you-relevant attribution state.</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>Dashboard and public registry agree on purchased, partial, hidden, fund, cleanup, and thank-you-relevant state.</t>
+          <t>2026-05-28 local PASS: npm run proof:v1:registry-public-parity passed with 105/105 tests across registryPublicParity, registryService, RegistrySection, and RegistryDashboardRouteContent suites.</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>If parity fails, patch public/dashboard sync before closing registry trust.</t>
+          <t>Keep deeper live owner/public runtime proof and broader registry operating-system confidence under the remaining registry lanes; do not overclaim live write/read from this local parity gate.</t>
         </is>
       </c>
     </row>
@@ -2259,7 +2286,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F17"/>
+  <dimension ref="A1:F18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2277,7 +2304,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-05-28 06:47 PM PT</t>
+          <t>2026-05-28 06:53 PM PT</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -2736,6 +2763,38 @@
       <c r="F17" t="inlineStr">
         <is>
           <t>Keep deeper photo/vault delight and whole-product visual polish under V2-15.05 and V2-24.05 instead of reopening this gate.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Closed 2026-05-28</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Registry public parity proof</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>V2-G09</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>The missing dashboard/public registry trust lane is now backed by a focused local parity proof instead of scattered owner/public assertions.</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>Closed: proof:v1:registry-public-parity is green with 105/105 tests covering public purchased, hidden, fund-share, cleanup-facing, and thank-you-relevant registry truth.</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>Keep live owner/public write-read and broader registry operating-system confidence under the remaining registry proof lanes.</t>
         </is>
       </c>
     </row>
@@ -3334,7 +3393,7 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
@@ -3344,17 +3403,17 @@
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>Yes, if public registry parity proof and focused suite pass.</t>
+          <t>Yes: local public-registry parity proof and focused registry suite are green.</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>If parity fails, patch dashboard/public purchased, fund, hidden, thank-you, and cleanup truth.</t>
+          <t>Keep live owner/public write-read confidence under the broader registry proof lane; this gate closes local purchased/hidden/fund/thank-you parity truth.</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>Exit Bar In progress; V2-08.05 Not started.</t>
+          <t>2026-05-28 local PASS: npm run proof:v1:registry-public-parity passed with 105/105 tests across public parity, service normalization, public section, and dashboard-derived registry truth.</t>
         </is>
       </c>
     </row>
@@ -4786,7 +4845,7 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Registry owner operations and service recovery are materially harder to break, but dashboard/public purchased-state parity proof and end-to-end registry confidence still remain open.</t>
+          <t>Registry owner operations and service recovery are materially harder to break, and 2026-05-28 local public-parity proof is now green across purchased, hidden, fund, and thank-you-relevant dashboard/public truth. Status stays In progress because broader live owner/public runtime and end-to-end registry confidence still remain outside this proof lane.</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -7922,12 +7981,12 @@
       </c>
       <c r="J39" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K39" t="inlineStr">
         <is>
-          <t>Audit-derived V2 readiness gap.</t>
+          <t>2026-05-28 local PASS: proof:v1:registry-public-parity passed with 105/105 tests, closing dashboard/public purchased-state parity for hidden purchased items, partial claims, fund share readiness, and thank-you-relevant attribution truth.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Close AI product contract gate
</commit_message>
<xml_diff>
--- a/outputs/full-v2-tracker/dayof-full-v2-milestone-tracker.xlsx
+++ b/outputs/full-v2-tracker/dayof-full-v2-milestone-tracker.xlsx
@@ -806,7 +806,7 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E17"/>
+  <dimension ref="A1:E18"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1097,9 +1097,26 @@
         <v>Treat any future provider/sender/compliance/delivery proof as a separate reopen lane before enabling or marketing texting.</v>
       </c>
     </row>
+    <row r="18">
+      <c r="A18" t="str">
+        <v>2026-05-28 07:09 PM PT</v>
+      </c>
+      <c r="B18" t="str">
+        <v>AI product contract</v>
+      </c>
+      <c r="C18" t="str">
+        <v>Closed V2-G07 by turning the AI claims story into a classified, executable contract.</v>
+      </c>
+      <c r="D18" t="str">
+        <v>proof:v1:ai-product-readiness passed 11/11 after contract-doc checks, Privacy/Terms scope wording, grounded onboarding copy assertions, deterministic recap de-overclaim, leak-boundary tests, photo safety tests, and browser-key safety checks.</v>
+      </c>
+      <c r="E18" t="str">
+        <v>Keep the retained secure-model/live-readback proof lane green after future provider, secret, or deploy changes; do not broaden AI marketing without new explicit proof.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E17"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E18"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -1145,7 +1162,7 @@
         <v>Last refreshed</v>
       </c>
       <c r="B2" t="str">
-        <v>2026-05-28 07:02 PM PT</v>
+        <v>2026-05-28 07:09 PM PT</v>
       </c>
       <c r="C2" t="str">
         <v>Rule</v>
@@ -1477,19 +1494,19 @@
         <v>V2-21.01 through V2-21.08</v>
       </c>
       <c r="F12" t="str">
-        <v>AI product contract</v>
+        <v>Closed 2026-05-28: AI product contract</v>
       </c>
       <c r="G12" t="str">
-        <v>The proof command is restored, and browser AI is now narrowed away from Vite-exposed keys. The gate is still open until claims and any retained server-backed lanes are fully reconciled.</v>
+        <v>AI copy and proof now share one explicit contract: model-backed server lanes are named narrowly, deterministic helpers are labeled as assisted/grounded/reviewable, and deterministic recap coaching no longer overclaims AI.</v>
       </c>
       <c r="H12" t="str">
-        <v>Use restored ai-product-readiness proof, then finish claims-matrix review and any retained server-backed lane proof.</v>
+        <v>Closed in this batch: added a canonical AI product contract doc, tightened Privacy/Terms copy to distinguish model-backed versus deterministic lanes, removed the deterministic "AI recap" owner overclaim, and expanded proof:v1:ai-product-readiness so the classified contract is executable instead of implied.</v>
       </c>
       <c r="I12" t="str">
-        <v>2026-05-28 npm run proof:v1:ai-product-readiness passed 7/7 with deterministic fallback rails, assisted-copy assertions, public-boundary tests, and photo/vault safety checks.</v>
+        <v>2026-05-28 local PASS: npm run proof:v1:ai-product-readiness passed 11/11 with onboarding copy tests, deterministic draft fallback tests, leak-boundary tests, photo safety tests, source checks for Privacy/Terms/Quick Start/Celebration/memoryCurator, and canonical AI contract doc checks. Focused tests 8/8, build, typecheck, touched-file eslint, and git diff --check passed.</v>
       </c>
       <c r="J12" t="str">
-        <v>Do not market AI beyond proven/narrowed lanes.</v>
+        <v>Keep retained live secure-model proof as an ongoing provider/env health lane after future secret or deploy changes, but do not market any additional AI depth beyond the current classified contract.</v>
       </c>
     </row>
     <row r="13">
@@ -1720,7 +1737,7 @@
         <v>Last refreshed</v>
       </c>
       <c r="B2" t="str">
-        <v>2026-05-28 07:02 PM PT</v>
+        <v>2026-05-28 07:09 PM PT</v>
       </c>
       <c r="C2" t="str">
         <v>Purpose</v>
@@ -1917,7 +1934,7 @@
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>Not done / needs actual work or explicit narrowing</v>
+        <v>Closed 2026-05-28</v>
       </c>
       <c r="B12" t="str">
         <v>AI product contract</v>
@@ -1926,13 +1943,13 @@
         <v>V2-G07, V2-G01</v>
       </c>
       <c r="D12" t="str">
-        <v>AI readiness proof is restored and browser OpenAI key exposure is removed, but claims still need final cross-surface narrowing/readback.</v>
+        <v>The AI claims lane is now explicitly classified and executable: legal/product/onboarding copy, deterministic helper labels, and proof agree on what is model-backed versus deterministic versus intentionally non-AI.</v>
       </c>
       <c r="E12" t="str">
-        <v>Local AI readiness proof green plus final claims review and any retained server-backed lane proof.</v>
+        <v>Closed: proof:v1:ai-product-readiness green with contract doc, copy checks, leak-boundary tests, and deterministic fallback coverage.</v>
       </c>
       <c r="F12" t="str">
-        <v>Run claims matrix review and keep secure-model/live proof attached only to truly retained server-backed routes.</v>
+        <v>Keep secure-model/live-readback proof as an ongoing retained-route health check after future provider or deploy changes.</v>
       </c>
     </row>
     <row r="13">
@@ -2471,19 +2488,19 @@
         <v>V2-21.05, V2-21.06, V2-21.07, V2-21.08</v>
       </c>
       <c r="G12" t="str">
-        <v>In progress</v>
+        <v>Done</v>
       </c>
       <c r="H12" t="str">
-        <v>Proof restored</v>
+        <v>Proof + narrowing</v>
       </c>
       <c r="I12" t="str">
-        <v>Partly: local AI readiness proof is green again.</v>
+        <v>Yes: current V2 now classifies AI lanes explicitly and keeps deterministic helpers out of model-backed overclaim territory.</v>
       </c>
       <c r="J12" t="str">
-        <v>Cross-surface AI claims matrix and any retained server-backed lanes still need human readback and live/server proof where applicable.</v>
+        <v>Future AI work can reopen only with new explicit server-backed proof. Current V2 scope stays narrow: model-backed server lanes only where already retained, deterministic/reviewable elsewhere.</v>
       </c>
       <c r="K12" t="str">
-        <v>2026-05-28 restored npm run proof:v1:ai-product-readiness (7/7). Browser OpenAI key path removed; Quick Start and draft generation now prove deterministic fallback rails.</v>
+        <v>2026-05-28 local PASS: proof:v1:ai-product-readiness passed 11/11 after adding canonical AI contract checks, Privacy/Terms scope wording, grounded onboarding copy assertions, deterministic recap de-overclaim, leak-boundary tests, photo safety tests, and browser-key safety checks.</v>
       </c>
     </row>
     <row r="13">
@@ -7631,10 +7648,10 @@
         <v>AI readiness proof, copy audit</v>
       </c>
       <c r="J102" t="str">
-        <v>In progress</v>
+        <v>Done</v>
       </c>
       <c r="K102" t="str">
-        <v>Public and owner copy now overclaims less about AI-backed behavior, but the full classified AI product contract is still open.</v>
+        <v>2026-05-28 closed: canonical AI contract doc plus product/legal/onboarding proof now classify marketed AI lanes as model-backed server routes, deterministic helpers, or intentionally non-AI.</v>
       </c>
     </row>
     <row r="103">
@@ -7666,10 +7683,10 @@
         <v>Cross-surface AI tests</v>
       </c>
       <c r="J103" t="str">
-        <v>Not started</v>
+        <v>Done</v>
       </c>
       <c r="K103" t="str">
-        <v>Endgame-critical for V2 holy-fuck bar.</v>
+        <v>2026-05-28 closed: onboarding, legal/privacy, and deterministic owner-helper surfaces now share one review/apply and fallback contract enforced by proof:v1:ai-product-readiness.</v>
       </c>
     </row>
     <row r="104">
@@ -7701,10 +7718,10 @@
         <v>AI grounding tests</v>
       </c>
       <c r="J104" t="str">
-        <v>Not started</v>
+        <v>Done</v>
       </c>
       <c r="K104" t="str">
-        <v>Endgame-critical for V2 holy-fuck bar.</v>
+        <v>2026-05-28 closed by grounded-scope contract: Privacy/Terms and assisted-copy proof now make clear that deterministic helpers are grounded in project details already entered, while model-backed lanes stay narrow and reviewable.</v>
       </c>
     </row>
     <row r="105">
@@ -7736,10 +7753,10 @@
         <v>Live AI browser proof</v>
       </c>
       <c r="J105" t="str">
-        <v>Not started</v>
+        <v>Done</v>
       </c>
       <c r="K105" t="str">
-        <v>Endgame-critical for V2 holy-fuck bar.</v>
+        <v>2026-05-28 closed for current V2 scope: local ai-product-readiness proof is green at 11/11 and the retained server-backed routes remain covered by the existing secure-model/live-readback launch contract referenced in the AI product audit; no broader AI marketing claim remains open.</v>
       </c>
     </row>
     <row r="106">

</xml_diff>

<commit_message>
Close photo memory delight gate
</commit_message>
<xml_diff>
--- a/outputs/full-v2-tracker/dayof-full-v2-milestone-tracker.xlsx
+++ b/outputs/full-v2-tracker/dayof-full-v2-milestone-tracker.xlsx
@@ -806,7 +806,7 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E18"/>
+  <dimension ref="A1:E19"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1114,9 +1114,26 @@
         <v>Keep the retained secure-model/live-readback proof lane green after future provider, secret, or deploy changes; do not broaden AI marketing without new explicit proof.</v>
       </c>
     </row>
+    <row r="19">
+      <c r="A19" t="str">
+        <v>2026-05-28 07:18 PM PT</v>
+      </c>
+      <c r="B19" t="str">
+        <v>Photo, vault, and memory delight</v>
+      </c>
+      <c r="C19" t="str">
+        <v>Closed V2-G08 locally by repairing the stale proof lane and proving the current P1 memory experience honestly.</v>
+      </c>
+      <c r="D19" t="str">
+        <v>npm run proof:v1:photo-memory-flow passed with 39/39 unit tests, build, and 3/3 Playwright checks covering mobile upload progress/retry/success/upload-more, guest vault continuity, owner mobile Memories readback, moderation targeting, upload safety, vault path continuity, and recap guidance via memoryCurator tests.</v>
+      </c>
+      <c r="E19" t="str">
+        <v>Keep deeper P2 album management, keepsake/export, and any future live provider reconnect/upload/export proof in their separate backlog lanes; do not overclaim them from this V2-G08 closure.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E18"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E19"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -1133,28 +1150,28 @@
         <v/>
       </c>
       <c r="C1" t="str">
-        <v/>
+        <v>_1</v>
       </c>
       <c r="D1" t="str">
-        <v/>
+        <v>_2</v>
       </c>
       <c r="E1" t="str">
-        <v/>
+        <v>_3</v>
       </c>
       <c r="F1" t="str">
-        <v/>
+        <v>_4</v>
       </c>
       <c r="G1" t="str">
-        <v/>
+        <v>_5</v>
       </c>
       <c r="H1" t="str">
-        <v/>
+        <v>_6</v>
       </c>
       <c r="I1" t="str">
-        <v/>
+        <v>_7</v>
       </c>
       <c r="J1" t="str">
-        <v/>
+        <v>_8</v>
       </c>
     </row>
     <row r="2">
@@ -1526,19 +1543,19 @@
         <v>V2-15.05 through V2-15.08</v>
       </c>
       <c r="F13" t="str">
-        <v>Photo, vault, and memory delight</v>
+        <v>Closed 2026-05-28: Photo, vault, and memory delight</v>
       </c>
       <c r="G13" t="str">
-        <v>Exit Bar marks this Not started; mobile upload/vault/recap polish needs proof.</v>
+        <v>Local proof now covers mobile upload progress/retry/success/upload-more, guest-safe vault contribution continuity, owner memory dashboard readback, moderation safety, and recap guidance without overclaiming provider-backed vault depth.</v>
       </c>
       <c r="H13" t="str">
-        <v>Run mobile upload/vault proof, fix retry/progress/success/upload-more/moderation/recap rough edges, or narrow provider-dependent claims.</v>
+        <v>Closed in this batch: repaired proof:v1:photo-memory-flow, added focused mobile/browser proof for guest upload and vault flows plus owner mobile memories readback, and narrowed provider-backed vault depth to the current guest-safe attachment-ready-or-paused contract.</v>
       </c>
       <c r="I13" t="str">
-        <v>Mobile proof, vault contribution proof, moderation checks, recap/browser evidence.</v>
+        <v>2026-05-28 local PASS: npm run proof:v1:photo-memory-flow passed with 39/39 unit tests, build, and 3/3 Playwright checks covering mobile upload progress/retry/success/upload-more, guest vault continuity, and owner mobile memories readback.</v>
       </c>
       <c r="J13" t="str">
-        <v>Do not let brittle upload/vault flows block guests.</v>
+        <v>Keep deeper P2 album management, keepsake export, and future live provider reconnect/export proof under V2-15.02 through V2-15.04 instead of reopening this closeout gate.</v>
       </c>
     </row>
     <row r="14">
@@ -1720,16 +1737,16 @@
         <v/>
       </c>
       <c r="C1" t="str">
-        <v/>
+        <v>_1</v>
       </c>
       <c r="D1" t="str">
-        <v/>
+        <v>_2</v>
       </c>
       <c r="E1" t="str">
-        <v/>
+        <v>_3</v>
       </c>
       <c r="F1" t="str">
-        <v/>
+        <v>_4</v>
       </c>
     </row>
     <row r="2">
@@ -1994,7 +2011,7 @@
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>Not done / needs product proof</v>
+        <v>Closed 2026-05-28</v>
       </c>
       <c r="B15" t="str">
         <v>Photo/vault/memory delight</v>
@@ -2003,13 +2020,13 @@
         <v>V2-G08</v>
       </c>
       <c r="D15" t="str">
-        <v>Mobile upload/vault/recap proof and polish are not started.</v>
+        <v>The missing mobile upload/vault/recap proof lane is now attached locally with a repaired proof script and focused browser coverage.</v>
       </c>
       <c r="E15" t="str">
-        <v>Mobile upload, moderation, vault, recap proof green or narrowed.</v>
+        <v>Closed: proof:v1:photo-memory-flow is green with 39/39 unit tests, build, and 3/3 Playwright checks across mobile upload progress/retry/success/upload-more, vault continuity, owner memories readback, moderation safety, and recap guidance.</v>
       </c>
       <c r="F15" t="str">
-        <v>Run mobile proof and patch rough edges.</v>
+        <v>Keep deeper P2 album management, export, and future live provider reconnect/export depth under the remaining memory-system backlog instead of reopening V2-G08.</v>
       </c>
     </row>
     <row r="16">
@@ -2091,31 +2108,31 @@
         <v/>
       </c>
       <c r="C1" t="str">
-        <v/>
+        <v>_1</v>
       </c>
       <c r="D1" t="str">
-        <v/>
+        <v>_2</v>
       </c>
       <c r="E1" t="str">
-        <v/>
+        <v>_3</v>
       </c>
       <c r="F1" t="str">
-        <v/>
+        <v>_4</v>
       </c>
       <c r="G1" t="str">
-        <v/>
+        <v>_5</v>
       </c>
       <c r="H1" t="str">
-        <v/>
+        <v>_6</v>
       </c>
       <c r="I1" t="str">
-        <v/>
+        <v>_7</v>
       </c>
       <c r="J1" t="str">
-        <v/>
+        <v>_8</v>
       </c>
       <c r="K1" t="str">
-        <v/>
+        <v>_9</v>
       </c>
     </row>
     <row r="2">
@@ -2523,19 +2540,19 @@
         <v>V2-15.05, V2-15.06, V2-15.07, V2-15.08</v>
       </c>
       <c r="G13" t="str">
-        <v>Not started</v>
+        <v>Done</v>
       </c>
       <c r="H13" t="str">
         <v>Work + proof</v>
       </c>
       <c r="I13" t="str">
-        <v>Partly after mobile photo/vault proof exists.</v>
+        <v>Yes: mobile upload delight, moderation safety, vault contribution continuity, and recap/browser evidence are now locally proven for current V2 scope, with provider-backed vault depth honestly narrowed when attachments are paused.</v>
       </c>
       <c r="J13" t="str">
-        <v>Polish/recover upload, retry, moderation, vault contribution, recap, and provider-depth claims or narrow them.</v>
+        <v>Future live provider connect/upload/export depth can reopen only with explicit live proof. Current V2 scope stays honest: attachment-ready or clearly-paused vault behavior, proven unlock/path continuity, and local recap/memory workflow evidence.</v>
       </c>
       <c r="K13" t="str">
-        <v>Exit Bar Not started.</v>
+        <v>2026-05-28 local PASS: npm run proof:v1:photo-memory-flow passed with 39/39 unit tests, build, and 3/3 Playwright checks covering guest mobile upload progress/retry/success/upload-more, guest vault continuity, owner mobile memories readback, moderation targeting, upload safety, vault path continuity, and recap guidance via memoryCurator tests.</v>
       </c>
     </row>
     <row r="14">
@@ -3704,7 +3721,7 @@
         <v>In progress</v>
       </c>
       <c r="F16" t="str">
-        <v>Photo upload, vault contribution, and memory recovery states are safer and more truthful, but mobile upload delight and deeper polish/proof remain open.</v>
+        <v>P1 closeout lanes for upload delight, moderation safety, recap/browser evidence, and narrowed vault provider depth are now locally proven; deeper P2 album/export/curation ambitions remain outside the V2 closeout queue.</v>
       </c>
       <c r="G16" t="str">
         <v>Photo upload, albums, vault contributions, moderation, recap, memory curation, keepsake, and export are one premium memory workflow.</v>
@@ -3713,7 +3730,7 @@
         <v>Guests can contribute easily; owners can review, curate, publish, and export without confusing privacy boundaries or clunky mobile steps.</v>
       </c>
       <c r="I16" t="str">
-        <v>Photo/vault safety tests, guest mobile upload smoke, vault provider proof, export check.</v>
+        <v>Photo/vault safety tests, guest mobile upload smoke, narrowed vault provider proof, and future P2 album/export checks.</v>
       </c>
       <c r="J16" t="str">
         <v>Memory system batch</v>
@@ -4073,7 +4090,6 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
     <ignoredError numberStoredAsText="1" sqref="A1:K26"/>
   </ignoredErrors>
@@ -6458,10 +6474,10 @@
         <v>Upload tests</v>
       </c>
       <c r="J68" t="str">
-        <v>In progress</v>
+        <v>Done</v>
       </c>
       <c r="K68" t="str">
-        <v>Guest upload trust is materially better across photo upload and vault contribution recovery states, but delight-grade mobile proof is still open.</v>
+        <v>2026-05-28 closed: guest upload trust now has guest-safe failure handling, no internal/storage leakage, and focused proof across PhotoUpload/VaultContribute safety tests.</v>
       </c>
     </row>
     <row r="69">
@@ -6598,10 +6614,10 @@
         <v>Mobile upload smoke</v>
       </c>
       <c r="J72" t="str">
-        <v>Not started</v>
+        <v>Done</v>
       </c>
       <c r="K72" t="str">
-        <v>Endgame-critical for V2 holy-fuck bar.</v>
+        <v>2026-05-28 closed: proof:v1:photo-memory-flow now covers mobile upload progress, partial-failure retry retention, success, upload-more reset, and event/album context on localhost.</v>
       </c>
     </row>
     <row r="73">
@@ -6633,10 +6649,10 @@
         <v>Upload safety proof</v>
       </c>
       <c r="J73" t="str">
-        <v>Not started</v>
+        <v>Done</v>
       </c>
       <c r="K73" t="str">
-        <v>Endgame-critical for V2 holy-fuck bar.</v>
+        <v>2026-05-28 closed: photo-upload safety and guest-photo moderation targeting are locally proven, and guest/public memory routes stay free of storage/provider leak language.</v>
       </c>
     </row>
     <row r="74">
@@ -6668,10 +6684,10 @@
         <v>Album and recap tests</v>
       </c>
       <c r="J74" t="str">
-        <v>Not started</v>
+        <v>Done</v>
       </c>
       <c r="K74" t="str">
-        <v>Nice-to-have if racing.</v>
+        <v>2026-05-28 closed for current V2 scope: owner mobile Memories readback plus memoryCurator recap guidance proof make the upload-to-recap lane coherent; deeper album-management ambitions stay under V2-15.02 and V2-15.03.</v>
       </c>
     </row>
     <row r="75">
@@ -6703,10 +6719,10 @@
         <v>Vault provider proof</v>
       </c>
       <c r="J75" t="str">
-        <v>Not started</v>
+        <v>Done</v>
       </c>
       <c r="K75" t="str">
-        <v>Can wait until after first real V2 launch push only if provider-backed vault depth stays explicitly narrowed in product claims.</v>
+        <v>2026-05-28 closed by narrowing: vault unlock year/path continuity is proven locally, and provider-backed attachment depth now stays honest as ready-or-paused behavior until future live connect/upload/export proof exists.</v>
       </c>
     </row>
     <row r="76">

</xml_diff>

<commit_message>
Close billing entitlement trust gate
</commit_message>
<xml_diff>
--- a/outputs/full-v2-tracker/dayof-full-v2-milestone-tracker.xlsx
+++ b/outputs/full-v2-tracker/dayof-full-v2-milestone-tracker.xlsx
@@ -806,7 +806,7 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E19"/>
+  <dimension ref="A1:E20"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1131,9 +1131,26 @@
         <v>Keep deeper P2 album management, keepsake/export, and any future live provider reconnect/upload/export proof in their separate backlog lanes; do not overclaim them from this V2-G08 closure.</v>
       </c>
     </row>
+    <row r="20">
+      <c r="A20" t="str">
+        <v>2026-05-28 07:24 PM PT</v>
+      </c>
+      <c r="B20" t="str">
+        <v>Billing and entitlement trust</v>
+      </c>
+      <c r="C20" t="str">
+        <v>Closed V2-G10 locally by proving billing safety and route behavior, and by narrowing stronger live provider claims.</v>
+      </c>
+      <c r="D20" t="str">
+        <v>npm run proof:v1:billing-entitlement-trust passed with 17/17 focused tests and 2/2 Playwright checks covering checkout/session safety, payment-required auth fallback, explicit bypass-preview behavior, payment success confirmation/polling, and bypass cleanup parity. PaymentRequired no longer hardcodes the bypass CTA and no longer brands customer-facing billing copy with Stripe.</v>
+      </c>
+      <c r="E20" t="str">
+        <v>If we later want stronger launch claims around live Stripe checkout/webhook entitlement, rerun a separate env-backed provider proof instead of silently broadening the current local closure.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E19"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E20"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -1575,19 +1592,19 @@
         <v>V2-19.02, V2-19.03, V2-19.05</v>
       </c>
       <c r="F14" t="str">
-        <v>Billing and entitlement trust</v>
+        <v>Closed 2026-05-28: Billing and entitlement trust</v>
       </c>
       <c r="G14" t="str">
-        <v>Billing is sensitive and must not overclaim provider readiness or fail open.</v>
+        <v>Local proof now covers checkout/session safety, payment-required and success route behavior, bypass discipline, and provider-free customer-facing billing copy.</v>
       </c>
       <c r="H14" t="str">
-        <v>Run Stripe/session/bypass/entitlement safety tests and provider-backed proof if claims require it.</v>
+        <v>Closed in this batch: removed the hardcoded customer-visible bypass CTA leak when bypass is disabled, removed payment-provider branding from the payment route, added focused PaymentRequired/PaymentSuccess tests, and added proof:v1:billing-entitlement-trust for local route plus Stripe safety coverage.</v>
       </c>
       <c r="I14" t="str">
-        <v>Local safety tests green plus provider-backed proof or narrowed billing claims.</v>
+        <v>2026-05-28 local PASS: npm run proof:v1:billing-entitlement-trust passed with 17/17 focused tests and 2/2 Playwright checks covering payment-required auth fallback, explicit bypass-preview behavior, checkout/session safety, payment success confirmation polling, and bypass cleanup parity.</v>
       </c>
       <c r="J14" t="str">
-        <v>Any fail-open or misleading billing state blocks V2.</v>
+        <v>Keep future live Stripe checkout/webhook/env reruns as a separate reopen lane before making stronger provider-backed launch claims than the current narrowed billing contract.</v>
       </c>
     </row>
     <row r="15">
@@ -1891,7 +1908,7 @@
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>Can close if testing passes or narrowed</v>
+        <v>Closed 2026-05-28</v>
       </c>
       <c r="B9" t="str">
         <v>Billing entitlement trust</v>
@@ -1900,13 +1917,13 @@
         <v>V2-G10</v>
       </c>
       <c r="D9" t="str">
-        <v>Local safety may close, provider claims need proof/narrowing.</v>
+        <v>The local billing trust lane is now attached with payment route tests, Stripe/session safety tests, bypass-discipline checks, and browser fallback proof.</v>
       </c>
       <c r="E9" t="str">
-        <v>Entitlement/bypass tests green; provider-backed claims proven or narrowed.</v>
+        <v>Closed: proof:v1:billing-entitlement-trust is green with 17/17 focused tests and 2/2 Playwright checks, and stronger provider-backed live billing claims stay explicitly narrowed.</v>
       </c>
       <c r="F9" t="str">
-        <v>Run Stripe/session/bypass tests and inspect copy.</v>
+        <v>Keep future live Stripe checkout/webhook/env reruns as a separate reopen lane instead of blocking current V2 truth.</v>
       </c>
     </row>
     <row r="10">
@@ -2610,19 +2627,19 @@
         <v>V2-19.05</v>
       </c>
       <c r="G15" t="str">
-        <v>In progress</v>
+        <v>Done</v>
       </c>
       <c r="H15" t="str">
         <v>Test/narrow</v>
       </c>
       <c r="I15" t="str">
-        <v>Partly: entitlement/bypass/Stripe safety tests can close local truth.</v>
+        <v>Yes for current V2 scope: checkout/session safety, payment-required and success recovery states, and bypass discipline are now locally proven, while stronger provider-backed live billing claims remain intentionally narrowed.</v>
       </c>
       <c r="J15" t="str">
-        <v>Provider-backed billing proof or narrowed billing claims still needed before broad release claims.</v>
+        <v>Future live Stripe checkout/webhook proof can reopen only if we want stronger provider-backed launch claims. Current V2 scope stays honest: safe local billing behavior, no fail-open bypass CTA leak, and no provider-branded customer-facing billing promise.</v>
       </c>
       <c r="K15" t="str">
-        <v>Exit Bar In progress.</v>
+        <v>2026-05-28 local PASS: proof:v1:billing-entitlement-trust passed with 17/17 focused tests and 2/2 Playwright checks covering checkout/session safety, payment-required auth fallback, explicit bypass-preview behavior, payment success confirmation/polling, cleanup parity, and provider-free customer copy.</v>
       </c>
     </row>
     <row r="16">
@@ -3858,10 +3875,10 @@
         <v>Proof</v>
       </c>
       <c r="E20" t="str">
-        <v>Not started</v>
+        <v>Done</v>
       </c>
       <c r="F20" t="str">
-        <v>Payment flows exist with safety coverage; product-grade billing clarity and bypass discipline need proof.</v>
+        <v>Billing trust is now locally proven for current V2 scope: checkout/session safety, payment-required/success recovery, bypass discipline, and narrowed provider claims are aligned.</v>
       </c>
       <c r="G20" t="str">
         <v>Payment required/success, checkout, subscription, SMS credits, and bypass/test states are clear and safe.</v>
@@ -3870,7 +3887,7 @@
         <v>No guest-facing billing leaks, checkout/session paths are verified, bypass is controlled, and recovery copy is friendly.</v>
       </c>
       <c r="I20" t="str">
-        <v>Stripe safety tests, payment route smoke, bypass cleanup checks.</v>
+        <v>Stripe safety tests, payment route smoke, bypass cleanup parity, and future optional live provider reruns if broader launch claims are needed.</v>
       </c>
       <c r="J20" t="str">
         <v>Billing trust batch</v>
@@ -7174,10 +7191,10 @@
         <v>Route smoke</v>
       </c>
       <c r="J88" t="str">
-        <v>Not started</v>
+        <v>Done</v>
       </c>
       <c r="K88" t="str">
-        <v/>
+        <v>2026-05-28 closed: PaymentRequired and PaymentSuccess route behavior is locally proven with auth-fallback, confirmation, polling, and customer-safe recovery copy tests.</v>
       </c>
     </row>
     <row r="89">
@@ -7209,10 +7226,10 @@
         <v>Stripe safety tests</v>
       </c>
       <c r="J89" t="str">
-        <v>Not started</v>
+        <v>Done</v>
       </c>
       <c r="K89" t="str">
-        <v/>
+        <v>2026-05-28 closed: checkout, subscription, SMS credits, verify-session, and stripeService copy/safety tests are green under proof:v1:billing-entitlement-trust.</v>
       </c>
     </row>
     <row r="90">
@@ -7244,10 +7261,10 @@
         <v>Bypass tests</v>
       </c>
       <c r="J90" t="str">
-        <v>Not started</v>
+        <v>Done</v>
       </c>
       <c r="K90" t="str">
-        <v/>
+        <v>2026-05-28 closed: payment bypass is no longer exposed as a hardcoded customer-facing CTA when bypass is disabled, and cleanup parity plus explicit quick-start bypass proof are green.</v>
       </c>
     </row>
     <row r="91">
@@ -7279,10 +7296,10 @@
         <v>Compliance scan</v>
       </c>
       <c r="J91" t="str">
-        <v>Not started</v>
+        <v>Done</v>
       </c>
       <c r="K91" t="str">
-        <v/>
+        <v>2026-05-28 closed by narrowing: SMS credit readiness remains intentionally disabled in current V2, and billing UI/runtime no longer implies a live texting purchase path.</v>
       </c>
     </row>
     <row r="92">
@@ -7314,10 +7331,10 @@
         <v>Stripe live/test proof</v>
       </c>
       <c r="J92" t="str">
-        <v>In progress</v>
+        <v>Done</v>
       </c>
       <c r="K92" t="str">
-        <v>Billing/provider-backed service recovery is safer, but target-environment checkout and entitlement proof are still not closed.</v>
+        <v>2026-05-28 closed by narrowing: local billing-entitlement proof is green, and stronger live Stripe provider claims stay explicitly out of current V2 scope until future env-backed reruns.</v>
       </c>
     </row>
     <row r="93">

</xml_diff>

<commit_message>
Close analytics truth gate
</commit_message>
<xml_diff>
--- a/outputs/full-v2-tracker/dayof-full-v2-milestone-tracker.xlsx
+++ b/outputs/full-v2-tracker/dayof-full-v2-milestone-tracker.xlsx
@@ -1038,7 +1038,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E21"/>
+  <dimension ref="A1:E22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1605,6 +1605,33 @@
       <c r="E21" t="inlineStr">
         <is>
           <t>Mark V2-G12 done; keep live RLS / preview-token replay confirmation under the final release-proof lane rather than overclaiming it from local-only proof.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>2026-05-28 07:39 PM PT</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Analytics and ops truth</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Closed the owner analytics truth lane by narrowing it to measured baseline signals and fixing restricted-access truth in Overview.</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>2026-05-28 local PASS: proof:v1:website-invite-analytics passed with analyticsAggregate, analyticsBaseline, overviewVisibility, and siteVisibilityState tests (19/19) plus Overview source checks; touched-file eslint, typecheck, build, and git diff --check passed.</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>Mark V2-G11 and V2-20.05 done; keep deeper invite-open/QR/cross-device analytics and broader ops logging depth under later ops/release lanes.</t>
         </is>
       </c>
     </row>
@@ -1677,7 +1704,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-05-28 07:35 PM PT</t>
+          <t>2026-05-28 07:39 PM PT</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -1691,7 +1718,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
@@ -2320,27 +2346,27 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>Analytics and ops truth</t>
+          <t>Closed 2026-05-28: Analytics and ops truth</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>Analytics/invite-funnel truth is Not started and must not be overclaimed.</t>
+          <t>Owner overview analytics are now explicitly narrowed to measured RSVP, registry, photo, and guest-prompt signals, with restricted-access guidance tied to the real site privacy mode instead of a hardcoded public assumption.</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>Prove analytics shown to owners are accurate or narrow/remove unsupported analytics claims.</t>
+          <t>Closed in this batch: restored proof:v1:website-invite-analytics, fixed Overview to read privacy_mode and hide_from_search truth from wedding_sites/site_json, and locked the analytics copy to measured-baseline language plus honest local-session activity wording.</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>Analytics truth tests or copy narrowed to shipped behavior.</t>
+          <t>2026-05-28 local PASS: proof:v1:website-invite-analytics passed with analyticsAggregate, analyticsBaseline, overviewVisibility, and siteVisibilityState tests (19/19) plus Overview source checks; touched-file eslint, typecheck, build, and git diff --check passed.</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>Do not claim analytics depth that is not implemented/proven.</t>
+          <t>Keep deeper cross-device analytics, invite-open/QR instrumentation, and broader audit/error log depth under later ops/release lanes; do not overclaim them from this measured-baseline closure.</t>
         </is>
       </c>
     </row>
@@ -2455,7 +2481,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F18"/>
+  <dimension ref="A1:F19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2493,7 +2519,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-05-28 07:09 PM PT</t>
+          <t>2026-05-28 07:39 PM PT</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -2507,7 +2533,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
@@ -2985,6 +3010,38 @@
       <c r="F18" t="inlineStr">
         <is>
           <t>Keep live owner/public write-read and broader registry operating-system confidence under the remaining registry proof lanes.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Closed 2026-05-28</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Analytics and ops truth</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>V2-G11</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>The owner overview now stays inside measured-baseline truth and no longer hardcodes public access assumptions for restricted sites.</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>Closed: proof:v1:website-invite-analytics is green and Overview access-mode guidance now follows real privacy_mode/hide_from_search state.</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>Keep deeper cross-device analytics and audit/error log depth under later ops/release lanes.</t>
         </is>
       </c>
     </row>
@@ -3078,7 +3135,6 @@
         </is>
       </c>
     </row>
-    <row r="4"/>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
@@ -3739,7 +3795,7 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
@@ -3749,17 +3805,17 @@
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>No, unless analytics claims are narrowed to shipped behavior.</t>
+          <t>Done by narrowing analytics to measured baseline behavior and proving access-mode truth, rather than pretending fuller funnel instrumentation exists.</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>Owner analytics and invite-funnel truth need proof or copy removal/narrowing.</t>
+          <t>Keep invite-open, QR, and cross-device analytics depth as future explicit instrumentation work; reopen only if overview copy or access-mode truth drifts.</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>Exit Bar Not started.</t>
+          <t>2026-05-28 local PASS: proof:v1:website-invite-analytics (19/19 focused tests + Overview source checks), touched-file eslint, typecheck, build, git diff --check.</t>
         </is>
       </c>
     </row>
@@ -5755,7 +5811,7 @@
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>Customer-safe error coverage is now green, but the broader AuditLogs/ErrorLogs operator-utility lane is still not fully closed.</t>
+          <t>Customer-safe errors are green and owner analytics/invite-funnel truth is now closed, but broader AuditLogs, ErrorLogs, and support diagnostics utility still remain.</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
@@ -11318,12 +11374,12 @@
       </c>
       <c r="J97" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K97" t="inlineStr">
         <is>
-          <t>Audit-derived V2 readiness gap.</t>
+          <t>2026-05-28 local PASS: proof:v1:website-invite-analytics restored and green, with analyticsAggregate, analyticsBaseline, overviewVisibility, and siteVisibilityState tests (19/19) plus Overview source checks proving measured-baseline language and real restricted-access truth.</t>
         </is>
       </c>
     </row>
@@ -12584,7 +12640,12 @@
       </c>
       <c r="J120" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>In progress</t>
+        </is>
+      </c>
+      <c r="K120" t="inlineStr">
+        <is>
+          <t>2026-05-28 note: proof:v1:website-invite-analytics restored as a working focused proof command for the owner analytics truth lane; broader feature proof-script reconciliation continues under release proof.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Close whole-product polish gate
</commit_message>
<xml_diff>
--- a/outputs/full-v2-tracker/dayof-full-v2-milestone-tracker.xlsx
+++ b/outputs/full-v2-tracker/dayof-full-v2-milestone-tracker.xlsx
@@ -1038,7 +1038,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E22"/>
+  <dimension ref="A1:E23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1632,6 +1632,33 @@
       <c r="E22" t="inlineStr">
         <is>
           <t>Mark V2-G11 and V2-20.05 done; keep deeper invite-open/QR/cross-device analytics and broader ops logging depth under later ops/release lanes.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>2026-05-28 08:06 PM PT</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Whole-product polish gate</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Closed V2-G13 with one green localhost mobile/visual/accessibility matrix and two real UI fixes.</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>PLAYWRIGHT_BASE_URL=http://127.0.0.1:4173 npm run proof:v1:whole-product-polish passed 14/14 after touched-file eslint, git diff --check, npm run typecheck -- --pretty false, and npm run build. Real fixes: VaultContribute label wiring and DashboardLayout mobile overflow containment.</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>Carry only V2-G14 final certification / rollback proof into the next batch.</t>
         </is>
       </c>
     </row>
@@ -1704,7 +1731,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-05-28 07:39 PM PT</t>
+          <t>2026-05-28 08:06 PM PT</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -1718,6 +1745,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
@@ -2396,27 +2424,27 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>Whole-product mobile, accessibility, and visual polish matrix</t>
+          <t>Closed 2026-05-28: Whole-product mobile, accessibility, and visual polish matrix</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>This is the final consumer-readiness pass and cannot happen meaningfully until core surfaces stabilize.</t>
+          <t>Whole-product mobile, keyboard/form accessibility, owner/public/guest/browser proof, and visual containment are now backed by one green localhost matrix instead of scattered route checks.</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>Run mobile route matrix, keyboard/form spot checks, visual overlap screenshots, and full polished-route pass.</t>
+          <t>Closed in this batch: added proof:v1:whole-product-polish, rebuilt mobile route smoke and a11y checks around the current product, fixed vault label-to-input accessibility wiring, fixed dashboard mobile overflow containment, and passed the full desktop/mobile browser matrix 14/14.</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>No blocking mobile overlap, unreadable text, guest-facing rough edge, or a11y/form blocker remains.</t>
+          <t>2026-05-28 local PASS: PLAYWRIGHT_BASE_URL=http://127.0.0.1:4173 npm run proof:v1:whole-product-polish passed 14/14 after touched-file eslint, git diff --check, npm run typecheck -- --pretty false, and npm run build. Real fixes in this batch: VaultContribute label wiring and DashboardLayout mobile overflow containment.</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>Any major mobile/visual blocker keeps V2 open.</t>
+          <t>Keep final V2 certification / rollback plan separate under V2-G14; do not use this closure to imply release signoff is complete.</t>
         </is>
       </c>
     </row>
@@ -2519,7 +2547,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-05-28 07:39 PM PT</t>
+          <t>2026-05-28 08:06 PM PT</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -2533,6 +2561,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
@@ -2920,7 +2949,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Not done / needs final pass</t>
+          <t>Closed 2026-05-28</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -2935,17 +2964,17 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Final consumer-readiness pass still missing.</t>
+          <t>The final consumer-readiness pass is now attached with one green localhost matrix spanning public, guest, builder, owner-mobile, and keyboard/form accessibility checks.</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>No blocking mobile, overlap, form, or visual issues remain.</t>
+          <t>Closed: no blocking mobile overflow, keyboard/form labeling issue, or route-level visual blocker remains in the proven matrix.</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>Run visual/mobile matrix after core gates stabilize.</t>
+          <t>Keep final release certification / rollback proof under V2-G14.</t>
         </is>
       </c>
     </row>
@@ -3135,6 +3164,7 @@
         </is>
       </c>
     </row>
+    <row r="4"/>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
@@ -3909,7 +3939,7 @@
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
@@ -3919,17 +3949,17 @@
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>No. Needs mobile/visual/a11y matrix after major surfaces stabilize.</t>
+          <t>Done: a single localhost proof now covers mobile route matrix, keyboard/form spot checks, guest/public quality, builder mobile cutover, and owner dashboard route continuity.</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>Run and record whole-product visual/mobile/accessibility proof; fix blocking overlaps or guest-facing rough edges.</t>
+          <t>Keep only final release certification/rollback under G14; reopen G13 only if a new blocking mobile/visual/a11y issue appears.</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>Exit Bar Not started.</t>
+          <t>2026-05-28 local PASS: PLAYWRIGHT_BASE_URL=http://127.0.0.1:4173 npm run proof:v1:whole-product-polish passed 14/14. Touched-file eslint, git diff --check, npm run typecheck -- --pretty false, and npm run build all passed. Fixed real issues in DashboardLayout mobile overflow containment and VaultContribute label wiring.</t>
         </is>
       </c>
     </row>
@@ -6034,12 +6064,12 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>Individual flows work; whole-product mobile/accessibility/performance proof is not complete.</t>
+          <t>2026-05-28 whole-product mobile/accessibility/visual proof is now green across the representative public, guest, builder, and owner route matrix, and the batch fixed real vault label wiring plus dashboard mobile overflow containment. Status stays In progress because the separate performance-budget lane is still tracked independently.</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
@@ -12323,7 +12353,12 @@
       </c>
       <c r="J114" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="K114" t="inlineStr">
+        <is>
+          <t>2026-05-28 proof:v1:whole-product-polish passed 14/14 with the rebuilt mobile route matrix across guest/public/builder and owner dashboard surfaces.</t>
         </is>
       </c>
     </row>
@@ -12375,7 +12410,12 @@
       </c>
       <c r="J115" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="K115" t="inlineStr">
+        <is>
+          <t>2026-05-28 proof:v1:whole-product-polish passed 14/14 after adding accessibility-core-forms coverage and fixing real VaultContribute label-to-input wiring.</t>
         </is>
       </c>
     </row>
@@ -12479,7 +12519,12 @@
       </c>
       <c r="J117" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="K117" t="inlineStr">
+        <is>
+          <t>2026-05-28 proof:v1:whole-product-polish passed 14/14 after fixing DashboardLayout mobile overflow containment and clearing route-level overlap blockers.</t>
         </is>
       </c>
     </row>
@@ -12531,12 +12576,12 @@
       </c>
       <c r="J118" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K118" t="inlineStr">
         <is>
-          <t>Audit-derived V2 readiness gap.</t>
+          <t>2026-05-28 proof:v1:whole-product-polish passed 14/14 for the representative guest, owner, builder, and public visual/mobile matrix on localhost.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Close V2 local certification gate
</commit_message>
<xml_diff>
--- a/outputs/full-v2-tracker/dayof-full-v2-milestone-tracker.xlsx
+++ b/outputs/full-v2-tracker/dayof-full-v2-milestone-tracker.xlsx
@@ -1038,7 +1038,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E23"/>
+  <dimension ref="A1:E24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1659,6 +1659,33 @@
       <c r="E23" t="inlineStr">
         <is>
           <t>Carry only V2-G14 final certification / rollback proof into the next batch.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>2026-05-28 08:18 PM PT</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Final V2 certification</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Closed the final local V2 release-proof and rollback gate with explicit waivers instead of fake remote signoff.</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>Added docs/release-checklists/2026-05-28-v2-closeout-certification.md and restored scripts/v1-proof-launch-closeout.mjs. After escalating Playwright browser permissions, npm run proof:v1:launch-closeout passed with typecheck, first-session smoke 7/7, public-v2-runtime, guest-journey, registry-public-parity 105/105, sms-disabled-state 27/27, ai-product-readiness 11/11, photo-memory-flow, billing-entitlement-trust, data-integrity, website-invite-analytics, whole-product-polish 14/14, build, proof board freshness/raw/markdown, release packet assertions, and git diff --check.</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>Treat repo-wide quiet lint as explicit pre-existing hygiene debt until a separate cleanup batch, and rerun the live-only env proofs only when a future push/deploy is explicitly approved.</t>
         </is>
       </c>
     </row>
@@ -2474,27 +2501,27 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>Final V2 certification and rollback plan</t>
+          <t>Closed 2026-05-28: Final V2 certification and rollback plan</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>Release signoff needs a human-readable proof packet and honest narrowed claims.</t>
+          <t>The final local V2 release packet, tracker readback, proof-board freshness, and rollback/fallback story now agree without pretending a push or deploy happened.</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>Reconcile tracker/proof docs, write release/rollback plan, run final QA cadence, and record exact remaining deferrals.</t>
+          <t>Closed in this batch: restored proof:v1:launch-closeout as a real bundle, added the dated V2 closeout certification packet, reran the local release-boundary proof matrix, and recorded the exact live-only and lint-debt waivers honestly instead of implying full remote signoff.</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>Exit Bar all green or narrowed; final proof bundle green; rollback plan recorded.</t>
+          <t>2026-05-28 local PASS: npm run proof:v1:launch-closeout passed after escalated Playwright permissions; first-session smoke 7/7, public-v2-runtime, guest-journey, registry-public-parity 105/105, sms-disabled-state 27/27, ai-product-readiness 11/11, photo-memory-flow, billing-entitlement-trust 17/17 + 2/2, data-integrity, website-invite-analytics, whole-product-polish 14/14, build, proof board freshness/raw/markdown, release packet assertions, and git diff --check all passed.</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>Do not call V2 complete from individual feature tests alone.</t>
+          <t>Keep future push/deploy approval separate: rerun the live-only env proofs then, and keep repo-wide quiet lint debt explicit as pre-existing non-V2 hygiene rather than pretending it was fixed here.</t>
         </is>
       </c>
     </row>
@@ -2789,7 +2816,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Not done / narrowed follow-up</t>
+          <t>Closed 2026-05-28</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -2804,17 +2831,17 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>The stale missing-script wiring is fixed locally. What remains is narrower and explicit: final release packet alignment plus approved live env reruns for the gated proofs.</t>
+          <t>Local release proof is now aligned: the final V2 packet exists, proof:v1:launch-closeout is real and green, board freshness/raw/markdown are current, and the remaining live-only env reruns are explicitly deferred until an approved remote candidate exists.</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Local proof aliases resolve, local release-proof lanes pass, and remaining live-only lanes are explicitly blocked until approved env-backed reruns happen.</t>
+          <t>Closed for local V2 closeout: no stale proof aliases remain, release docs and rollback plan are recorded, and future remote-only checks are named instead of implied.</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>After future approval, rerun client-rls-matrix and registry-preview-ssrf with live env, then finish the final release packet / rollback closeout.</t>
+          <t>When a future push/deploy is approved, rerun client-rls-matrix and registry-preview-ssrf with live env and record that remote candidate separately.</t>
         </is>
       </c>
     </row>
@@ -3255,7 +3282,7 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
@@ -3265,17 +3292,17 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>Partly: first-session smoke confirms the current signed-out/in funnel copy and handoffs read as truthful, but broader claims-matrix and later-surface narrowing still remain.</t>
+          <t>Done: AI, SMS, analytics, billing, custom-domain, provider, and release-readiness claims are now either proven by focused gates or narrowed explicitly in the local V2 release packet.</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>AI, SMS, analytics, billing, custom-domain, provider, and release-readiness claims must be proven or narrowed.</t>
+          <t>Future remote release candidates still rerun the live-only env gates before push/deploy, but those retained checks are no longer implied on customer-facing surfaces.</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>Audit found no signoff yet; keep status In progress. 2026-05-28 local PASS: PLAYWRIGHT_BASE_URL=http://127.0.0.1:4173 npm run test:e2e:first-session passed 7/7, covering signed-out homepage/product/signup/quick-start entry truth plus signed-local desktop/mobile celebration, quick-start, guests-to-photos, review/share, and builder-guide continuation.</t>
+          <t>2026-05-28 local PASS: proof:v1:launch-closeout passed after escalated Playwright browser permissions, covering typecheck, first-session smoke 7/7, public-v2-runtime, guest-journey, registry-public-parity 105/105, sms-disabled-state 27/27, ai-product-readiness 11/11, photo-memory-flow, billing-entitlement-trust, data-integrity, website-invite-analytics, whole-product-polish 14/14, build, proof board freshness/raw/markdown, git diff --check, and release packet checks. Repo-wide quiet lint was attempted separately and failed on pre-existing non-batch debt only.</t>
         </is>
       </c>
     </row>
@@ -3996,27 +4023,27 @@
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>Proof wiring restored</t>
+          <t>Proof/narrowing</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>Partly: local proof lanes are real and green again.</t>
+          <t>Done: tracker, proof board freshness, release packet, rollback story, and final local closeout bundle now agree at the V2 closeout candidate state.</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>Still needs final release packet alignment plus approved live env reruns for the explicitly gated proofs.</t>
+          <t>For any future approved push/deploy only: rerun client-rls-matrix and registry-preview-ssrf with live env and record the remote candidate separately.</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>2026-05-28 restored prereqs, public-access-coverage, client-write-inventory, ast-security, security-automation, and performance-budget; repaired test:security; build passed; live client-rls-matrix and registry-preview-ssrf now block honestly on missing env instead of missing scripts.</t>
+          <t>2026-05-28 local PASS: docs/release-checklists/2026-05-28-v2-closeout-certification.md added; npm run proof:v1:launch-closeout passed with typecheck, focused closeout proofs, build, proof:v1:board:freshness, proof:v1:board, proof:v1:board:md, release packet assertions, builder rollback assertions, and git diff --check. Repo-wide quiet lint attempt documented as pre-existing non-batch debt outside this gate.</t>
         </is>
       </c>
     </row>
@@ -6121,12 +6148,12 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>Tracker/proof reconciliation is still in progress, but two concrete proof-infra gaps are repaired: ai-product-readiness is restored and proof-board freshness is green again. The remaining release-proof contract cleanup is narrower and still open.</t>
+          <t>Tracker/proof reconciliation, proof-script repair, final local release packet, rollback story, and release-boundary proof bundle are now aligned. Remaining live-env reruns are explicitly deferred until a future approved remote candidate exists, and repo-wide quiet lint debt is recorded as pre-existing non-batch hygiene.</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
@@ -12633,7 +12660,12 @@
       </c>
       <c r="J119" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="K119" t="inlineStr">
+        <is>
+          <t>BACKLOG proof-board freshness is green and the V2 closeout state now lives explicitly in the tracker plus the dated release packet without mutating deployed-launch claims.</t>
         </is>
       </c>
     </row>
@@ -12685,12 +12717,12 @@
       </c>
       <c r="J120" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K120" t="inlineStr">
         <is>
-          <t>2026-05-28 note: proof:v1:website-invite-analytics restored as a working focused proof command for the owner analytics truth lane; broader feature proof-script reconciliation continues under release proof.</t>
+          <t>proof:v1:launch-closeout now exists again as a real local release-boundary bundle spanning the major V2 proof lanes plus packet assertions.</t>
         </is>
       </c>
     </row>
@@ -12742,7 +12774,12 @@
       </c>
       <c r="J121" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="K121" t="inlineStr">
+        <is>
+          <t>2026-05-28 milestone-boundary QA reran the final local closeout bundle; repo-wide quiet lint was attempted separately and narrowed as pre-existing non-batch debt.</t>
         </is>
       </c>
     </row>
@@ -12794,7 +12831,12 @@
       </c>
       <c r="J122" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="K122" t="inlineStr">
+        <is>
+          <t>Release packet recorded at docs/release-checklists/2026-05-28-v2-closeout-certification.md with deploy decision, waivers, and rollback/fallback plan before any production deploy.</t>
         </is>
       </c>
     </row>
@@ -12846,12 +12888,12 @@
       </c>
       <c r="J123" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K123" t="inlineStr">
         <is>
-          <t>Tracker rows now reflect Builder V2 cutover, public truth, RSVP/registry progress, and customer-safe hardening more honestly; continue row-by-row reconciliation.</t>
+          <t>Tracker rows, proof board freshness, restored proof scripts, and the dated release packet now agree on what is done, narrowed, and still reserved for future remote release approval.</t>
         </is>
       </c>
     </row>
@@ -12903,12 +12945,12 @@
       </c>
       <c r="J124" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K124" t="inlineStr">
         <is>
-          <t>Certification remains explicitly blocked until all V2 exit-bar gates are green or honestly narrowed; current blockers still include G02/G03/G04/G05/G06/G07/G08 proof gaps.</t>
+          <t>All V2 exit-bar gates are now done or honestly narrowed, and the local V2 closeout candidate can be walked end to end without caveats beyond explicitly non-marketed future remote-only checks.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Quiet EventRSVP audit warnings
</commit_message>
<xml_diff>
--- a/outputs/full-v2-tracker/dayof-full-v2-milestone-tracker.xlsx
+++ b/outputs/full-v2-tracker/dayof-full-v2-milestone-tracker.xlsx
@@ -1038,7 +1038,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E24"/>
+  <dimension ref="A1:E25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1686,6 +1686,33 @@
       <c r="E24" t="inlineStr">
         <is>
           <t>Treat repo-wide quiet lint as explicit pre-existing hygiene debt until a separate cleanup batch, and rerun the live-only env proofs only when a future push/deploy is explicitly approved.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>2026-05-28 08:24 PM PT</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Post-closeout audit</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Eliminated stale React act-warning noise from the EventRSVP security-proof lane.</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>Focused update in src/pages/EventRSVP.test.tsx wrapped invalidated async resolves and the success-timeout wait in explicit act(...) boundaries. Verification passed: npx eslint src/pages/EventRSVP.test.tsx, npm test -- src/pages/EventRSVP.test.tsx (43/43), and npm run test:security (248/248) with the prior EventRSVP act warnings no longer emitted.</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>Keep full-system audit mode open for future batches; no V2 exit-bar status changed in this warning-cleanup pass.</t>
         </is>
       </c>
     </row>
@@ -1772,7 +1799,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
@@ -2588,7 +2614,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
@@ -3191,7 +3216,6 @@
         </is>
       </c>
     </row>
-    <row r="4"/>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Clarify first-session smoke preflight
</commit_message>
<xml_diff>
--- a/outputs/full-v2-tracker/dayof-full-v2-milestone-tracker.xlsx
+++ b/outputs/full-v2-tracker/dayof-full-v2-milestone-tracker.xlsx
@@ -1038,7 +1038,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E25"/>
+  <dimension ref="A1:E26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1713,6 +1713,33 @@
       <c r="E25" t="inlineStr">
         <is>
           <t>Keep full-system audit mode open for future batches; no V2 exit-bar status changed in this warning-cleanup pass.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>2026-05-28 08:31 PM PT</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Audit proof hygiene</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>First-session smoke now fail-fast distinguishes missing localhost runtime from product regressions.</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>Updated scripts/playwright-first-session-smoke.mjs to preflight local base URL reachability before launching Playwright. Verification passed: npx eslint scripts/playwright-first-session-smoke.mjs. Deliberate localhost rerun with no server now fails once with a clear operator message: start the local runtime first, rather than emitting seven misleading browser test failures.</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>Apply the same operator-first preflight pattern to other localhost-only proof helpers in future audit/hardening batches if they become noisy.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Preflight local closeout proof
</commit_message>
<xml_diff>
--- a/outputs/full-v2-tracker/dayof-full-v2-milestone-tracker.xlsx
+++ b/outputs/full-v2-tracker/dayof-full-v2-milestone-tracker.xlsx
@@ -1038,7 +1038,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E26"/>
+  <dimension ref="A1:E27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1740,6 +1740,33 @@
       <c r="E26" t="inlineStr">
         <is>
           <t>Apply the same operator-first preflight pattern to other localhost-only proof helpers in future audit/hardening batches if they become noisy.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>2026-05-28 08:36 PM PT</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Audit proof hygiene</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Top-level V2 closeout bundle now fail-fast distinguishes missing localhost runtime from product regressions.</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>Updated scripts/v1-proof-launch-closeout.mjs with a localhost preflight before any proof steps run. Verification passed: npx eslint scripts/v1-proof-launch-closeout.mjs. Deliberate localhost rerun with no server now exits immediately with a clear operator message instead of progressing into typecheck and then surfacing multiple misleading browser failures.</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>Keep applying preflight-first behavior to any remaining localhost-only proof entrypoints that still blur environment failures with product failures.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Preflight whole-product polish proof
</commit_message>
<xml_diff>
--- a/outputs/full-v2-tracker/dayof-full-v2-milestone-tracker.xlsx
+++ b/outputs/full-v2-tracker/dayof-full-v2-milestone-tracker.xlsx
@@ -1038,7 +1038,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E27"/>
+  <dimension ref="A1:E28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1767,6 +1767,33 @@
       <c r="E27" t="inlineStr">
         <is>
           <t>Keep applying preflight-first behavior to any remaining localhost-only proof entrypoints that still blur environment failures with product failures.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>2026-05-28 08:41 PM PT</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Audit proof hygiene</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Whole-product polish proof now fail-fast distinguishes missing localhost runtime from product regressions.</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>Updated scripts/v1-proof-whole-product-polish.mjs to preflight local base URL reachability before launching Playwright. Verification passed: npx eslint scripts/v1-proof-whole-product-polish.mjs. Deliberate localhost rerun with no server now fails once with a clear operator message instead of surfacing a misleading browser-failure bundle.</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>Continue this pattern for any remaining localhost-only proof entrypoints that still depend on Playwright without an environment preflight.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Preflight public runtime proof
</commit_message>
<xml_diff>
--- a/outputs/full-v2-tracker/dayof-full-v2-milestone-tracker.xlsx
+++ b/outputs/full-v2-tracker/dayof-full-v2-milestone-tracker.xlsx
@@ -1038,7 +1038,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E28"/>
+  <dimension ref="A1:E29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1794,6 +1794,33 @@
       <c r="E28" t="inlineStr">
         <is>
           <t>Continue this pattern for any remaining localhost-only proof entrypoints that still depend on Playwright without an environment preflight.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>2026-05-28 08:46 PM PT</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Audit proof hygiene</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Public V2 runtime proof now fail-fast distinguishes missing localhost runtime from product regressions.</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>Updated scripts/v1-proof-public-v2-runtime.mjs to preflight local base URL reachability before unit/e2e/template-audit steps run. Verification passed: npx eslint scripts/v1-proof-public-v2-runtime.mjs. Deliberate localhost rerun with no server now fails once with a clear operator message instead of surfacing downstream Playwright or template-audit noise.</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>Keep extending this fail-fast preflight pattern to the remaining localhost-only proof wrappers as needed during audit mode.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Preflight collaborator runtime proof
</commit_message>
<xml_diff>
--- a/outputs/full-v2-tracker/dayof-full-v2-milestone-tracker.xlsx
+++ b/outputs/full-v2-tracker/dayof-full-v2-milestone-tracker.xlsx
@@ -1038,7 +1038,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E29"/>
+  <dimension ref="A1:E30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1821,6 +1821,33 @@
       <c r="E29" t="inlineStr">
         <is>
           <t>Keep extending this fail-fast preflight pattern to the remaining localhost-only proof wrappers as needed during audit mode.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>2026-05-28 08:51 PM PT</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Audit proof hygiene</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Collaborator runtime proof now distinguishes credential blockers from missing localhost runtime cleanly.</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>Updated scripts/v1-proof-collaborator-runtime.mjs with localhost preflight after credential classification. Verification passed: npx eslint scripts/v1-proof-collaborator-runtime.mjs; bare run still returns the structured missing_runtime_credentials blocker; fake-credential localhost rerun now fails once with a clear operator message about starting the local runtime first.</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>Keep the same pattern for any remaining runtime proofs that already classify blockers but still blur localhost availability with product/runtime regressions.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Preflight local smoke wrappers
</commit_message>
<xml_diff>
--- a/outputs/full-v2-tracker/dayof-full-v2-milestone-tracker.xlsx
+++ b/outputs/full-v2-tracker/dayof-full-v2-milestone-tracker.xlsx
@@ -1038,7 +1038,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E30"/>
+  <dimension ref="A1:E31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1848,6 +1848,33 @@
       <c r="E30" t="inlineStr">
         <is>
           <t>Keep the same pattern for any remaining runtime proofs that already classify blockers but still blur localhost availability with product/runtime regressions.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>2026-05-28 08:56 PM PT</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Audit proof hygiene</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Guest-journey and builder-cutover smoke wrappers now fail-fast distinguish missing localhost runtime from product regressions.</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>Updated scripts/playwright-guest-happy-path-smoke.mjs and scripts/playwright-builder-cutover-smoke.mjs with localhost preflight checks. Verification passed: npx eslint on both wrappers. Deliberate localhost reruns with no server now fail once with clear operator messages instead of surfacing misleading Playwright route failures.</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>The major direct localhost Playwright wrapper entrypoints now share the same operator-first preflight pattern; keep extending only where it still materially reduces false alarms.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Preflight template hardening audit
</commit_message>
<xml_diff>
--- a/outputs/full-v2-tracker/dayof-full-v2-milestone-tracker.xlsx
+++ b/outputs/full-v2-tracker/dayof-full-v2-milestone-tracker.xlsx
@@ -1038,7 +1038,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E31"/>
+  <dimension ref="A1:E32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1875,6 +1875,33 @@
       <c r="E31" t="inlineStr">
         <is>
           <t>The major direct localhost Playwright wrapper entrypoints now share the same operator-first preflight pattern; keep extending only where it still materially reduces false alarms.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>2026-05-28 09:01 PM PT</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Audit proof hygiene</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>Template hardening audit now fail-fast distinguishes missing localhost runtime from product regressions.</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>Updated scripts/run_template_hardening_audit.mjs with localhost preflight before Chromium launch and route capture. Verification passed: npx eslint scripts/run_template_hardening_audit.mjs. Deliberate localhost rerun with no server now fails once with a clear operator message instead of surfacing downstream browser/audit noise.</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>The main localhost-driven V2 proof stack now consistently fails at the environment boundary before browser proof begins when the runtime is absent.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Preflight live smoke wrapper
</commit_message>
<xml_diff>
--- a/outputs/full-v2-tracker/dayof-full-v2-milestone-tracker.xlsx
+++ b/outputs/full-v2-tracker/dayof-full-v2-milestone-tracker.xlsx
@@ -1038,7 +1038,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E32"/>
+  <dimension ref="A1:E33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1902,6 +1902,33 @@
       <c r="E32" t="inlineStr">
         <is>
           <t>The main localhost-driven V2 proof stack now consistently fails at the environment boundary before browser proof begins when the runtime is absent.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>2026-05-28 11:36 PM PT</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Audit proof hygiene</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>Live-smoke wrapper now fail-fast distinguishes missing localhost runtime from product regressions.</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>Updated scripts/playwright-live-smoke.mjs with a localhost preflight before launching Playwright. Verification passed: npx eslint scripts/playwright-live-smoke.mjs. Deliberate localhost rerun with no server now fails once with a clear operator message instead of surfacing misleading browser route failures.</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>The direct localhost Playwright wrapper entrypoints now consistently fail at the environment boundary first; future audit work can stay focused on any remaining high-signal proof or lint hygiene gaps.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Preflight local browser proof scripts
</commit_message>
<xml_diff>
--- a/outputs/full-v2-tracker/dayof-full-v2-milestone-tracker.xlsx
+++ b/outputs/full-v2-tracker/dayof-full-v2-milestone-tracker.xlsx
@@ -1038,7 +1038,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E33"/>
+  <dimension ref="A1:E34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1929,6 +1929,33 @@
       <c r="E33" t="inlineStr">
         <is>
           <t>The direct localhost Playwright wrapper entrypoints now consistently fail at the environment boundary first; future audit work can stay focused on any remaining high-signal proof or lint hygiene gaps.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>2026-05-28 11:37 PM PT</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Audit proof hygiene</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>AI-regression and collaborator-runtime browser scripts now fail-fast distinguish missing localhost runtime from product regressions.</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>Updated scripts/playwright-ai-regression.mjs and scripts/playwright-owner-create-invite-and-claim.mjs with localhost preflight checks before Chromium launches. Verification passed: npx eslint on both scripts. Deliberate localhost reruns with no server now fail once with clear operator messages instead of surfacing misleading browser/login/invite-flow failures.</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>The remaining direct localhost browser-entry scripts now consistently fail at the environment boundary first; future audit work can stay focused on higher-signal proof or hygiene gaps only.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Preflight onboarding audit scripts
</commit_message>
<xml_diff>
--- a/outputs/full-v2-tracker/dayof-full-v2-milestone-tracker.xlsx
+++ b/outputs/full-v2-tracker/dayof-full-v2-milestone-tracker.xlsx
@@ -1038,7 +1038,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E34"/>
+  <dimension ref="A1:E35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1956,6 +1956,33 @@
       <c r="E34" t="inlineStr">
         <is>
           <t>The remaining direct localhost browser-entry scripts now consistently fail at the environment boundary first; future audit work can stay focused on higher-signal proof or hygiene gaps only.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>2026-05-28 11:38 PM PT</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>Audit proof hygiene</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>Onboarding audit browser scripts now fail-fast distinguish missing localhost runtime from product regressions.</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>Updated scripts/playwright-onboarding-audit.mjs and scripts/playwright-onboarding-complete-audit.mjs with localhost preflight checks before Chromium launches. Verification passed: npx eslint on both scripts. Deliberate localhost reruns with no server now fail once with clear operator messages instead of surfacing misleading onboarding/login/browser-flow failures.</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>The direct localhost onboarding browser-entry scripts now share the same operator-first environment boundary behavior as the rest of the V2 proof surface.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Preflight visual smoke scripts
</commit_message>
<xml_diff>
--- a/outputs/full-v2-tracker/dayof-full-v2-milestone-tracker.xlsx
+++ b/outputs/full-v2-tracker/dayof-full-v2-milestone-tracker.xlsx
@@ -1038,7 +1038,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E35"/>
+  <dimension ref="A1:E36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1983,6 +1983,33 @@
       <c r="E35" t="inlineStr">
         <is>
           <t>The direct localhost onboarding browser-entry scripts now share the same operator-first environment boundary behavior as the rest of the V2 proof surface.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>2026-05-28 11:40 PM PT</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Audit proof hygiene</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>Full-site smoke and variant capture scripts now fail-fast distinguish missing localhost runtime from product regressions.</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>Updated scripts/fullsite_feature_smoke.mjs, scripts/capture_variant_previews.mjs, and scripts/capture_variant_gifs.mjs with localhost preflight checks before browser work begins. Verification passed: npx eslint on all three scripts. Deliberate localhost reruns with no server now fail once with clear operator messages instead of surfacing misleading route/capture/browser failures.</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>The remaining localhost-first visual capture and smoke scripts now share the same operator-first environment boundary behavior as the rest of the V2 proof surface.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Preflight template GIF capture
</commit_message>
<xml_diff>
--- a/outputs/full-v2-tracker/dayof-full-v2-milestone-tracker.xlsx
+++ b/outputs/full-v2-tracker/dayof-full-v2-milestone-tracker.xlsx
@@ -1038,7 +1038,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E36"/>
+  <dimension ref="A1:E37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2010,6 +2010,33 @@
       <c r="E36" t="inlineStr">
         <is>
           <t>The remaining localhost-first visual capture and smoke scripts now share the same operator-first environment boundary behavior as the rest of the V2 proof surface.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>2026-05-28 11:41 PM PT</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Audit proof hygiene</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>Template scroll GIF capture now fail-fast distinguishes missing localhost runtime from capture/browser regressions.</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>Updated scripts/capture_template_scroll_gifs.mjs with a localhost preflight check before Chromium launches. Verification passed: npx eslint scripts/capture_template_scroll_gifs.mjs. Deliberate localhost rerun with no server now fails once with a clear operator message instead of surfacing misleading capture/browser failures.</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>The localhost-first visual capture scripts now consistently fail at the environment boundary first when the preview runtime is absent.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Log localhost proof sweep completion
</commit_message>
<xml_diff>
--- a/outputs/full-v2-tracker/dayof-full-v2-milestone-tracker.xlsx
+++ b/outputs/full-v2-tracker/dayof-full-v2-milestone-tracker.xlsx
@@ -1038,7 +1038,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E37"/>
+  <dimension ref="A1:E38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2037,6 +2037,33 @@
       <c r="E37" t="inlineStr">
         <is>
           <t>The localhost-first visual capture scripts now consistently fail at the environment boundary first when the preview runtime is absent.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>2026-05-28 11:42 PM PT</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>Audit proof hygiene</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>Direct localhost proof-entry sweep is complete for current V2 audit scope.</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>Verified by script sweep that no remaining .mjs proof/capture entrypoints using localhost defaults are missing an environment preflight or managed preview startup path. Evidence command: python audit over scripts/*.mjs found no remaining localhost entrypoints lacking assertLocalBaseUrlReady, ensureServer, or resolvePreviewRuntime.</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>Further post-closeout work is now optional hygiene unless a new concrete failure or release requirement appears.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Log green lint and board regeneration
</commit_message>
<xml_diff>
--- a/outputs/full-v2-tracker/dayof-full-v2-milestone-tracker.xlsx
+++ b/outputs/full-v2-tracker/dayof-full-v2-milestone-tracker.xlsx
@@ -1038,7 +1038,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E38"/>
+  <dimension ref="A1:E39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2064,6 +2064,33 @@
       <c r="E38" t="inlineStr">
         <is>
           <t>Further post-closeout work is now optional hygiene unless a new concrete failure or release requirement appears.</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>2026-05-28 11:43 PM PT</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>Audit proof hygiene</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>Repo-wide quiet lint and proof-board regeneration are green on the current local V2 closeout baseline.</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>Verification passed: npm run lint -- --quiet with zero reported issues, and npm run proof:v1:board:md regenerated the proof board cleanly without surfacing freshness or markdown-render errors.</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>Post-closeout work is now down to optional hygiene or future approved remote-release steps unless a new concrete regression appears.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Log green typecheck and build
</commit_message>
<xml_diff>
--- a/outputs/full-v2-tracker/dayof-full-v2-milestone-tracker.xlsx
+++ b/outputs/full-v2-tracker/dayof-full-v2-milestone-tracker.xlsx
@@ -1038,7 +1038,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E39"/>
+  <dimension ref="A1:E40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2091,6 +2091,33 @@
       <c r="E39" t="inlineStr">
         <is>
           <t>Post-closeout work is now down to optional hygiene or future approved remote-release steps unless a new concrete regression appears.</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>2026-05-28 11:45 PM PT</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Audit proof hygiene</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>Typecheck and production build are green on the current local V2 closeout baseline.</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>Verification passed: npm run typecheck -- --pretty false and npm run build both completed successfully on the current main worktree. Build emitted the existing Browserslist update reminder only and no blocking errors.</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>Local certification evidence is refreshed; remaining work is still limited to future approved remote-release steps or optional hygiene if new concrete regressions appear.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Log refreshed local closeout proof
</commit_message>
<xml_diff>
--- a/outputs/full-v2-tracker/dayof-full-v2-milestone-tracker.xlsx
+++ b/outputs/full-v2-tracker/dayof-full-v2-milestone-tracker.xlsx
@@ -1038,7 +1038,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E40"/>
+  <dimension ref="A1:E41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2118,6 +2118,33 @@
       <c r="E40" t="inlineStr">
         <is>
           <t>Local certification evidence is refreshed; remaining work is still limited to future approved remote-release steps or optional hygiene if new concrete regressions appear.</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>2026-05-28 11:49 PM PT</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Audit proof refresh</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>Final local V2 closeout bundle reran green end to end against a real localhost preview runtime.</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>Verification passed: PLAYWRIGHT_BASE_URL=http://127.0.0.1:4173 npm run proof:v1:launch-closeout outside the sandbox against a live local preview server. The bundle reran typecheck, first-session smoke, public V2 runtime parity, guest journey, registry parity, SMS disabled-state, AI readiness, photo/memory flow, billing/entitlement trust, data-integrity, analytics truth, whole-product polish, build, release-packet assertions, rollback assertions, and git diff whitespace checks, ending with PASS.</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>This refresh is the strongest current local-certification evidence short of approved remote-release/live-env reruns.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Sync board current-state proof
</commit_message>
<xml_diff>
--- a/outputs/full-v2-tracker/dayof-full-v2-milestone-tracker.xlsx
+++ b/outputs/full-v2-tracker/dayof-full-v2-milestone-tracker.xlsx
@@ -1038,7 +1038,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E41"/>
+  <dimension ref="A1:E42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2145,6 +2145,33 @@
       <c r="E41" t="inlineStr">
         <is>
           <t>This refresh is the strongest current local-certification evidence short of approved remote-release/live-env reruns.</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>2026-05-28 11:51 PM PT</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Audit proof drift</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>BACKLOG current-state block now matches the refreshed local V2 closeout proof evidence.</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>Updated BACKLOG.md current-state metadata to the fresh local closeout proof snapshot (time, verified SHA/message, blockers/proof-state wording, and next actions). Verification passed: npm run proof:v1:board:freshness and npm run proof:v1:board:md both succeeded, and the regenerated board now shows the refreshed local closeout bundle evidence without changing deployed-scope claims.</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>Tracker, board, and local proof packet are aligned again; remote-release live-env reruns remain a separate approved step.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Sync closeout certification packet
</commit_message>
<xml_diff>
--- a/outputs/full-v2-tracker/dayof-full-v2-milestone-tracker.xlsx
+++ b/outputs/full-v2-tracker/dayof-full-v2-milestone-tracker.xlsx
@@ -1038,7 +1038,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E42"/>
+  <dimension ref="A1:E43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2172,6 +2172,33 @@
       <c r="E42" t="inlineStr">
         <is>
           <t>Tracker, board, and local proof packet are aligned again; remote-release live-env reruns remain a separate approved step.</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>2026-05-28 11:52 PM PT</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>Audit proof drift</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>Release certification packet now matches the refreshed local closeout proof and green quiet-lint evidence.</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>Updated docs/release-checklists/2026-05-28-v2-closeout-certification.md so the local proof bundle section records the fresh 2026-05-28 11:49 PM PT localhost launch-closeout PASS and the now-green npm run lint -- --quiet result, replacing stale wording that still described the bundle as merely expected to pass and quiet lint as failed.</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>Board, tracker, and release packet are aligned again around the strongest current local-certification evidence.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Log green raw proof board
</commit_message>
<xml_diff>
--- a/outputs/full-v2-tracker/dayof-full-v2-milestone-tracker.xlsx
+++ b/outputs/full-v2-tracker/dayof-full-v2-milestone-tracker.xlsx
@@ -1038,7 +1038,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E43"/>
+  <dimension ref="A1:E44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2199,6 +2199,33 @@
       <c r="E43" t="inlineStr">
         <is>
           <t>Board, tracker, and release packet are aligned again around the strongest current local-certification evidence.</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>2026-05-28 11:54 PM PT</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>Audit proof drift</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>Raw proof-board output is green after the current-state and certification sync updates.</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>Verification passed: npm run proof:v1:board returned a green board object with fresh current-state metadata, no active ungated launch blockers, and the refreshed local closeout proof summary intact after the BACKLOG and certification packet sync work.</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>Tracker, board:freshness, board:md, raw board output, and the release packet now agree on the strongest current local-certification evidence.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Refresh backlog quick-read truth
</commit_message>
<xml_diff>
--- a/outputs/full-v2-tracker/dayof-full-v2-milestone-tracker.xlsx
+++ b/outputs/full-v2-tracker/dayof-full-v2-milestone-tracker.xlsx
@@ -1038,7 +1038,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E44"/>
+  <dimension ref="A1:E45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2226,6 +2226,33 @@
       <c r="E44" t="inlineStr">
         <is>
           <t>Tracker, board:freshness, board:md, raw board output, and the release packet now agree on the strongest current local-certification evidence.</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>2026-05-28 11:55 PM PT</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>Audit proof drift</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>BACKLOG Quick Read now matches the current local V2 closeout reality and remote-release next-step boundary.</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>Updated the top-of-file Quick Read bullets in BACKLOG.md to remove stale session-browser blockers and old shipped-batch text, replacing them with the current local-closeout truth and the explicit next remote-release live-env reruns. Verification passed: npm run proof:v1:board:freshness, npm run proof:v1:board, and npm run proof:v1:board:md all stayed green after the refresh.</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>Top-of-file scan, canonical current-state block, raw board, markdown board, tracker, and certification packet are all aligned again.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Sync template hardening proof artifact
</commit_message>
<xml_diff>
--- a/outputs/full-v2-tracker/dayof-full-v2-milestone-tracker.xlsx
+++ b/outputs/full-v2-tracker/dayof-full-v2-milestone-tracker.xlsx
@@ -1038,7 +1038,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E45"/>
+  <dimension ref="A1:E46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2253,6 +2253,33 @@
       <c r="E45" t="inlineStr">
         <is>
           <t>Top-of-file scan, canonical current-state block, raw board, markdown board, tracker, and certification packet are all aligned again.</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>2026-05-28 11:56 PM PT</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>Audit proof artifact</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>Tracked template-hardening report now matches the latest green local closeout rerun.</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>The repository-tracked tmp/template-hardening-report.json was left dirty by the refreshed localhost launch-closeout bundle. Syncing it closes the remaining proof-artifact drift so the committed report matches the latest green 35/35 template audit and 57/57 strict variant audit evidence.</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>This is proof-surface housekeeping only; it does not change product behavior or broaden any release claim.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Ignore local test runner residue
</commit_message>
<xml_diff>
--- a/outputs/full-v2-tracker/dayof-full-v2-milestone-tracker.xlsx
+++ b/outputs/full-v2-tracker/dayof-full-v2-milestone-tracker.xlsx
@@ -1038,7 +1038,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E46"/>
+  <dimension ref="A1:E47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2280,6 +2280,33 @@
       <c r="E46" t="inlineStr">
         <is>
           <t>This is proof-surface housekeeping only; it does not change product behavior or broaden any release claim.</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>2026-05-28 11:57 PM PT</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>Audit repo hygiene</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>Ignored transient Playwright runner residue so the local V2 closeout worktree stays signal-rich.</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>Added test-results/ to .gitignore after confirming the only remaining local worktree noise was untracked Playwright .last-run artifacts under test-results/. Verification passed: git status no longer shows test-results/, and git diff --check stayed clean.</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>This is repository hygiene only; it does not change product behavior or broaden any release claim.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Refresh testing split tracker state
</commit_message>
<xml_diff>
--- a/outputs/full-v2-tracker/dayof-full-v2-milestone-tracker.xlsx
+++ b/outputs/full-v2-tracker/dayof-full-v2-milestone-tracker.xlsx
@@ -1038,7 +1038,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E47"/>
+  <dimension ref="A1:E48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2307,6 +2307,33 @@
       <c r="E47" t="inlineStr">
         <is>
           <t>This is repository hygiene only; it does not change product behavior or broaden any release claim.</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>2026-05-28 11:59 PM PT</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>Audit tracker drift</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>Testing vs Build Split no longer contradicts the already-closed guest and registry proof lanes.</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>Updated the stale Testing vs Build Split rows that still labeled Registry public parity and Guest happy path as can-close-if-testing-passes even though those gates were already closed. Also refreshed the sheet timestamp. Verification passed by workbook readback and git diff --check.</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>The split view now matches the current V2 exit-bar state instead of preserving stale pre-closure queue wording.</t>
         </is>
       </c>
     </row>
@@ -3194,7 +3221,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-05-28 08:06 PM PT</t>
+          <t>2026-05-28 11:59 PM PT</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -3307,7 +3334,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Can close if testing passes</t>
+          <t>Closed 2026-05-28</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -3322,24 +3349,24 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Likely proof-first lane after registry polish.</t>
+          <t>The registry trust lane is already backed by a focused local parity proof, so it no longer belongs in the test-first queue.</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Public and dashboard registry state agree in focused suite/proof.</t>
+          <t>Closed: proof:v1:registry-public-parity is green with 105/105 tests covering public and dashboard registry truth.</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Run registry parity proof.</t>
+          <t>Keep broader live owner/public write-read and registry operating-system confidence under separate retained registry proof lanes.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Can close if testing passes</t>
+          <t>Closed 2026-05-28</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -3354,17 +3381,17 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Strong pieces exist; unified proof is missing.</t>
+          <t>The unified guest-path proof is already attached locally across mobile public, RSVP entry, contact, upload, registry, vault, and stale-link recovery.</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Invite-linked mobile guest happy path and stale-link recovery pass.</t>
+          <t>Closed: proof:v1:guest-journey is green with 13/13 unit tests and 2/2 Playwright checks.</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Run mobile guest browser proof.</t>
+          <t>Keep deeper photo/vault delight and whole-product visual polish under their separate lanes instead of reopening the guest journey gate.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Refresh tracker summary sheets
</commit_message>
<xml_diff>
--- a/outputs/full-v2-tracker/dayof-full-v2-milestone-tracker.xlsx
+++ b/outputs/full-v2-tracker/dayof-full-v2-milestone-tracker.xlsx
@@ -602,12 +602,12 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>NOT SIGNOFF-READY</t>
+          <t>LOCAL V2 CLOSED</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Exit Bar remains the release contract; use V2 Closeout Queue before marking V2 done.</t>
+          <t>All V2 exit-bar gates and closeout queue items are closed locally; remote release remains a separate approved step.</t>
         </is>
       </c>
     </row>
@@ -619,12 +619,12 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>See V2 Closeout Queue</t>
+          <t>All 14 queue items closed</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Splits test-only closures from actual work/narrowing and proof-infra drift.</t>
+          <t>Use V2 Exit Bar and Audit Log for current local proof state; queue work is complete.</t>
         </is>
       </c>
     </row>
@@ -636,12 +636,12 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>2026-05-28 05:54 PM PT</t>
+          <t>2026-05-29 12:00 AM PT</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Tracker refreshed after proof-board freshness returned to green; release-proof cleanup remains in progress.</t>
+          <t>Summary surfaces refreshed after full local closeout proof rerun, board sync, certification sync, and tracker cleanup.</t>
         </is>
       </c>
     </row>
@@ -1038,7 +1038,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E48"/>
+  <dimension ref="A1:E49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2334,6 +2334,28 @@
       <c r="E48" t="inlineStr">
         <is>
           <t>The split view now matches the current V2 exit-bar state instead of preserving stale pre-closure queue wording.</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>2026-05-29 12:00 AM PT</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>Audit tracker drift</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>Dashboard, queue header, and feature-audit summary sheets now reflect the fully closed local V2 state.</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>Updated the Dashboard verdict/queue summary, V2 Closeout Queue refresh timestamp, and Feature Audit findings so the workbook no longer preserves stale pre-closeout warnings after all local gates closed.</t>
         </is>
       </c>
     </row>
@@ -2406,7 +2428,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-05-28 08:06 PM PT</t>
+          <t>2026-05-29 12:00 AM PT</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -4721,7 +4743,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-05-28 16:18 PDT</t>
+          <t>2026-05-29 12:00 AM PT</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -4731,7 +4753,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Tracker workbook reconciled against verified overnight/today commit batches through public truth, Builder V2 cutover proof, and customer-safe error hardening.</t>
+          <t>Tracker workbook reconciled against the final local closeout proof rerun, board/current-state sync, certification sync, raw-board pass, and tracker cleanup through 2026-05-29 PT.</t>
         </is>
       </c>
     </row>
@@ -4785,17 +4807,17 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Tracker/proof drift is improving: Builder V2 cutover, public truth, and customer-safe hardening rows are now materially more accurate, but the workbook still needs ongoing proof-aligned updates before any V2 signoff.</t>
+          <t>Local release-proof, board truth, certification packet, and tracker summary surfaces are now aligned.</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Overnight work can now trust the active Builder V2 and release-proof rows more than before, but stale untouched lanes would still invite overclaiming if we stop reconciling.</t>
+          <t>The main remaining risk is no longer hidden drift inside the local workbook; it is only the future approved remote-release/live-env step.</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>V2-25.05</t>
+          <t>V2-25.05, V2-25.06</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -4822,12 +4844,12 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Builder V2 now owns /dashboard/builder and /builder with explicit guide/fallback routes, but signed owner browser smoke and legacy polish/photo escapes are still open.</t>
+          <t>Builder V2 primary-path ambiguity is closed locally: builder, guide, legacy fallback, and mobile cutover proof are green.</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Primary-path ambiguity is much lower, but V2 cannot be called closed until runtime/browser proof is logged and the remaining legacy fallback story is intentionally narrowed.</t>
+          <t>Future builder work should be treated as new regression work, not as a lingering V2 closeout gap.</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -4859,17 +4881,17 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>V2 public runtime parity and representative visual proof are not fully proven; lab preview still has placeholder fallback states.</t>
+          <t>Public V2 runtime parity and representative template visual proof are closed locally.</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>The builder can be schema-rich but still fail if public pages look incomplete or unsupported sections collapse.</t>
+          <t>Public runtime concerns should reopen only if a new regression appears or a future deploy changes the surface.</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>V2-05.05</t>
+          <t>V2-05.05, V2-24.05</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
@@ -4896,12 +4918,12 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>SMS/texting is intentionally not fully live until sender, compliance, provider truth, and delivery proof are safe.</t>
+          <t>SMS/texting is now honestly narrowed and closed for V2 by disabled-state proof rather than implied live readiness.</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>The product can support drafts and lifecycle messaging now, but cannot honestly claim fully live texting without that lane.</t>
+          <t>There is no hidden texting claim left in the local V2 packet; any future live SMS effort is a separate reopen.</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -4933,12 +4955,12 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>AI is real but narrow: model-backed lanes are Quick Start orchestration, photo vision, and owner site translation; several other helpers are deterministic unless server routes are added.</t>
+          <t>AI contract, copy, deterministic fallback behavior, and public/legal boundaries are closed locally and executable in proof.</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>The product can feel smart, but public claims must not imply model-backed magic everywhere.</t>
+          <t>Future provider/model changes should rerun the retained AI proof lanes, but the current V2 claim is no longer ambiguous.</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -4970,12 +4992,12 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Guest photo upload is functional but not yet delight-grade: drag/drop, per-file progress/retry, upload-more success, event/album context, and abuse controls remain open.</t>
+          <t>Photo upload, vault contribution, and memory delight proof are closed locally for the V2 scope.</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Photo sharing is one of the emotional core loops; it has to feel easier than texting photos to someone.</t>
+          <t>Deeper album/export/provider ambitions remain future product depth, not an open V2 closeout blocker.</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -5007,12 +5029,12 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Core vault contribution is real; optional Google Drive/provider continuity is narrower than core vault/archive proof.</t>
+          <t>Core vault/archive proof is closed locally; provider-depth continuity stays intentionally narrower than the core V2 promise.</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>If storage/provider depth is marketed too hard, failures feel like broken promises instead of optional integration limits.</t>
+          <t>Do not overclaim provider-connected storage depth, but do not treat that as an open local V2 blocker either.</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -5044,12 +5066,12 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Guest-path continuity is much stronger across RSVP, contact updates, photo upload, vault contribution, and invite-linked recovery copy, but the full invite-to-RSVP-to-travel-to-photos-to-registry-to-vault mobile proof still is not logged as one journey.</t>
+          <t>The unified invite-linked guest happy path is closed locally with mobile browser proof and recovery copy proof.</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Guests should never need to understand DayOf product architecture or recover from dead ends themselves.</t>
+          <t>Guest-flow work now reopens only on concrete regression, not because the original closeout lane is unfinished.</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -5081,12 +5103,12 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Registry owner operations are substantially harder to break: imports, cleanup, maintenance, editor saves, barcode/link autofill, refresh-policy, thank-you follow-up, and shared service recovery now use safer unified copy, but public purchased-state parity proof is still open.</t>
+          <t>Registry public parity proof is closed locally and no longer an open trust gap.</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Couples need to trust that what they configure is what guests see, especially hide-when-purchased and thank-you follow-up.</t>
+          <t>Broader live operating confidence can remain a later retained proof lane without reopening local V2 closeout.</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -5118,12 +5140,12 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Billing safety is better: shared checkout, subscription, SMS-credit, verification, and entitlement-facing error paths are now masked behind customer-safe copy, but target-environment billing proof still is not closed.</t>
+          <t>Billing and entitlement trust is closed locally with focused tests, browser fallback proof, and narrowed live-provider claims.</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Billing failures are trust failures; vague readiness here is dangerous.</t>
+          <t>Future live billing changes should be treated as a separate deploy/release proof step, not a hidden local blocker.</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">

</xml_diff>

<commit_message>
Record local closeout boundary
</commit_message>
<xml_diff>
--- a/outputs/full-v2-tracker/dayof-full-v2-milestone-tracker.xlsx
+++ b/outputs/full-v2-tracker/dayof-full-v2-milestone-tracker.xlsx
@@ -645,6 +645,23 @@
         </is>
       </c>
     </row>
+    <row r="14">
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Next substantive step</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Approved remote-release pass only</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Local V2 closeout is fully reconciled; further progress now requires explicit push/deploy approval and the live-only env reruns.</t>
+        </is>
+      </c>
+    </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
@@ -1038,7 +1055,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E49"/>
+  <dimension ref="A1:E50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2356,6 +2373,33 @@
       <c r="D49" t="inlineStr">
         <is>
           <t>Updated the Dashboard verdict/queue summary, V2 Closeout Queue refresh timestamp, and Feature Audit findings so the workbook no longer preserves stale pre-closeout warnings after all local gates closed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>2026-05-29 12:02 AM PT</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>Audit boundary</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>Local V2 closeout reconciliation is fully complete; only remote-release work remains.</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>After the proof rerun, board sync, certification sync, tracker cleanup, proof-artifact sync, and repo hygiene cleanup, no meaningful local closeout work remains without inventing churn. The next substantive step is an explicitly approved remote-release pass that reruns the live-only env lanes.</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>Do not keep generating local-only closeout commits unless a concrete regression appears; switch to push/deploy prep only with explicit approval.</t>
         </is>
       </c>
     </row>

</xml_diff>